<commit_message>
Group D: the user's 6 Brennan STEPs settle Q1-Q4 - 66 of 68 bent tubes generate (tube wider than hub ends flat, 6701-04/-06 own neck, 6701-20-20 M 3.26); closed loop vs 11 STEPs, 66/66 all-config OK
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ef5oeTLN9TDbfPmJS2gewx
</commit_message>
<xml_diff>
--- a/tools/_out/groupD_20261021/regen/stage/DesignTable_1704T_SW2.xlsx
+++ b/tools/_out/groupD_20261021/regen/stage/DesignTable_1704T_SW2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA34"/>
+  <dimension ref="A1:BA36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="AZ7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-16-16: L1 3.39 L2 2.6 AF 1.375 JT 0.453 GT 0.911 AFL 1.75 EFL 0.315 BFL 1.56 DFL 1.496 FFL 0.551 DRILLFL 0.75 TOD 1.043 EXT 2.026 (codes: README s2). </t>
+          <t>Brennan record 1704-16-16: L1 3.39 L2 2.6 AF 1.375 JT 0.453 GT 0.911 AFL 1.75 EFL 0.315 BFL 1.56 DFL 1.496 FFL 0.551 DRILLFL 0.75 TOD 1.043 EXT 2.026 (codes: README s2).  BRENNAN_1704-16-16.stp: torus R 1.6208 = 0.8 x EXT 2.026 (second STEP size of the 90 deg bend rule), tube 1.043 / 0.750.</t>
         </is>
       </c>
       <c r="BA7" t="inlineStr">
@@ -2193,7 +2193,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1704-20-16-Tube</t>
+          <t>1704-20-12-Tube</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2257,70 +2257,70 @@
         <v>0.957952</v>
       </c>
       <c r="V10" t="n">
-        <v>1.9008</v>
+        <v>1.8016</v>
       </c>
       <c r="W10" t="n">
-        <v>1.6392</v>
+        <v>1.2504</v>
       </c>
       <c r="X10" t="n">
-        <v>3.54</v>
+        <v>3.052</v>
       </c>
       <c r="Y10" t="n">
-        <v>2.099</v>
+        <v>1.709</v>
       </c>
       <c r="Z10" t="n">
         <v>1.339</v>
       </c>
       <c r="AA10" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB10" t="n">
         <v>0.625</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>0.78</v>
       </c>
       <c r="AC10" t="n">
         <v>0.11</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.875</v>
+        <v>0.75</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.315</v>
+        <v>0.265</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.748</v>
+        <v>0.63</v>
       </c>
       <c r="AG10" t="n">
         <v>0.551</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.501</v>
+        <v>0.551</v>
       </c>
       <c r="AI10" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ10" t="n">
-        <v>1.9008</v>
+        <v>1.8016</v>
       </c>
       <c r="AK10" t="n">
-        <v>1.6392</v>
+        <v>1.2504</v>
       </c>
       <c r="AL10" t="n">
-        <v>3.54</v>
+        <v>3.052</v>
       </c>
       <c r="AM10" t="n">
-        <v>2.65</v>
+        <v>2.31</v>
       </c>
       <c r="AN10" t="n">
         <v>0.75</v>
       </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>1704-20-16-Tube</t>
+          <t>1704-20-12-Tube</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -16</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -12</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
@@ -2335,22 +2335,22 @@
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -16 (O 1.75)</t>
+          <t>SAE code 61 flange head -12 (O 1.5)</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>3.540</t>
+          <t>3.052</t>
         </is>
       </c>
       <c r="AU10" t="inlineStr">
         <is>
-          <t>2.600</t>
+          <t>2.260</t>
         </is>
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>1.639</t>
+          <t>1.250</t>
         </is>
       </c>
       <c r="AW10" t="inlineStr">
@@ -2365,24 +2365,24 @@
       </c>
       <c r="AY10" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-16 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-12 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled); the tube is wider than the hub and ends flat at its back face (as on BRENNAN_1704-20-12.stp)</t>
         </is>
       </c>
       <c r="AZ10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-20-16: L1 3.54 L2 2.6 AF 1.6875 JT 0.531 GT 0.958 AFL 1.75 EFL 0.315 BFL 1.56 DFL 1.496 FFL 0.551 DRILLFL 0.75 TOD 1.339 EXT 2.049 (codes: README s2). </t>
+          <t>Brennan record 1704-20-12: L1 3.052 L2 2.26 AF 1.6875 JT 0.531 GT 0.958 AFL 1.5 EFL 0.265 BFL 1.25 DFL 1.26 FFL 0.551 DRILLFL 0.75 TOD 1.339 EXT 1.563 (codes: README s2).  BRENNAN_1704-20-12.stp confirms the record: the 1.339 tube is wider than the 1.260 hub and ends flat at the hub back face (y -1.709); R 1.2504 = 0.8 x EXT.</t>
         </is>
       </c>
       <c r="BA10" t="inlineStr">
         <is>
-          <t>1704-20-16-Tube</t>
+          <t>1704-20-12-Tube</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1704-20-20-Tube</t>
+          <t>1704-20-16-Tube</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2446,37 +2446,37 @@
         <v>0.957952</v>
       </c>
       <c r="V11" t="n">
-        <v>1.9968</v>
+        <v>1.9008</v>
       </c>
       <c r="W11" t="n">
-        <v>1.9832</v>
+        <v>1.6392</v>
       </c>
       <c r="X11" t="n">
-        <v>3.98</v>
+        <v>3.54</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.529</v>
+        <v>2.099</v>
       </c>
       <c r="Z11" t="n">
         <v>1.339</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.72</v>
+        <v>0.625</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.875</v>
+        <v>0.78</v>
       </c>
       <c r="AC11" t="n">
         <v>0.11</v>
       </c>
       <c r="AD11" t="n">
-        <v>1</v>
+        <v>0.875</v>
       </c>
       <c r="AE11" t="n">
         <v>0.315</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.8465</v>
+        <v>0.748</v>
       </c>
       <c r="AG11" t="n">
         <v>0.551</v>
@@ -2488,28 +2488,28 @@
         <v>0.05</v>
       </c>
       <c r="AJ11" t="n">
-        <v>1.9968</v>
+        <v>1.9008</v>
       </c>
       <c r="AK11" t="n">
-        <v>1.9832</v>
+        <v>1.6392</v>
       </c>
       <c r="AL11" t="n">
-        <v>3.98</v>
+        <v>3.54</v>
       </c>
       <c r="AM11" t="n">
-        <v>3.08</v>
+        <v>2.65</v>
       </c>
       <c r="AN11" t="n">
-        <v>1.004</v>
+        <v>0.75</v>
       </c>
       <c r="AO11" t="inlineStr">
         <is>
-          <t>1704-20-20-Tube</t>
+          <t>1704-20-16-Tube</t>
         </is>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -20</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -16</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
@@ -2524,22 +2524,22 @@
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -20 (O 2)</t>
+          <t>SAE code 61 flange head -16 (O 1.75)</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>3.980</t>
+          <t>3.540</t>
         </is>
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>3.030</t>
+          <t>2.600</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>1.983</t>
+          <t>1.639</t>
         </is>
       </c>
       <c r="AW11" t="inlineStr">
@@ -2554,24 +2554,24 @@
       </c>
       <c r="AY11" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-20 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-16 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-20-20: L1 3.98 L2 3.03 AF 1.6875 JT 0.531 GT 0.958 AFL 2.0 EFL 0.315 BFL 1.75 DFL 1.693 FFL 0.551 DRILLFL 1.004 TOD 1.339 EXT 2.479 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1704-20-16: L1 3.54 L2 2.6 AF 1.6875 JT 0.531 GT 0.958 AFL 1.75 EFL 0.315 BFL 1.56 DFL 1.496 FFL 0.551 DRILLFL 0.75 TOD 1.339 EXT 2.049 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA11" t="inlineStr">
         <is>
-          <t>1704-20-20-Tube</t>
+          <t>1704-20-16-Tube</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1704-20-24-Tube</t>
+          <t>1704-20-20-Tube</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2635,70 +2635,70 @@
         <v>0.957952</v>
       </c>
       <c r="V12" t="n">
-        <v>1.996</v>
+        <v>1.9968</v>
       </c>
       <c r="W12" t="n">
-        <v>1.984</v>
+        <v>1.9832</v>
       </c>
       <c r="X12" t="n">
         <v>3.98</v>
       </c>
       <c r="Y12" t="n">
-        <v>2.53</v>
+        <v>2.529</v>
       </c>
       <c r="Z12" t="n">
         <v>1.339</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.9025</v>
+        <v>0.72</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.0575</v>
+        <v>0.875</v>
       </c>
       <c r="AC12" t="n">
         <v>0.11</v>
       </c>
       <c r="AD12" t="n">
-        <v>1.1875</v>
+        <v>1</v>
       </c>
       <c r="AE12" t="n">
         <v>0.315</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.9845</v>
+        <v>0.8465</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.63</v>
+        <v>0.551</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.58</v>
+        <v>0.501</v>
       </c>
       <c r="AI12" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ12" t="n">
-        <v>1.996</v>
+        <v>1.9968</v>
       </c>
       <c r="AK12" t="n">
-        <v>1.984</v>
+        <v>1.9832</v>
       </c>
       <c r="AL12" t="n">
         <v>3.98</v>
       </c>
       <c r="AM12" t="n">
-        <v>3.16</v>
+        <v>3.08</v>
       </c>
       <c r="AN12" t="n">
         <v>1.004</v>
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>1704-20-24-Tube</t>
+          <t>1704-20-20-Tube</t>
         </is>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -24</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -20</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -24 (O 2.375)</t>
+          <t>SAE code 61 flange head -20 (O 2)</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
@@ -2723,12 +2723,12 @@
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>3.110</t>
+          <t>3.030</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>1.984</t>
+          <t>1.983</t>
         </is>
       </c>
       <c r="AW12" t="inlineStr">
@@ -2743,31 +2743,31 @@
       </c>
       <c r="AY12" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-24 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-20 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-20-24: L1 3.98 L2 3.11 AF 1.6875 JT 0.531 GT 0.958 AFL 2.375 EFL 0.315 BFL 2.12 DFL 1.969 FFL 0.63 DRILLFL 1.004 TOD 1.339 EXT 2.480 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1704-20-20: L1 3.98 L2 3.03 AF 1.6875 JT 0.531 GT 0.958 AFL 2.0 EFL 0.315 BFL 1.75 DFL 1.693 FFL 0.551 DRILLFL 1.004 TOD 1.339 EXT 2.479 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA12" t="inlineStr">
         <is>
-          <t>1704-20-24-Tube</t>
+          <t>1704-20-20-Tube</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1704-20-32-Tube</t>
+          <t>1704-20-24-Tube</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>1.488952</v>
       </c>
       <c r="C13" t="n">
-        <v>0.974567</v>
+        <v>0.974279</v>
       </c>
       <c r="D13" t="n">
         <v>0.8125</v>
@@ -2812,7 +2812,7 @@
         <v>0.08333</v>
       </c>
       <c r="R13" t="n">
-        <v>1.688</v>
+        <v>1.6875</v>
       </c>
       <c r="S13" t="n">
         <v>0.957952</v>
@@ -2824,37 +2824,37 @@
         <v>0.957952</v>
       </c>
       <c r="V13" t="n">
-        <v>1.9864</v>
+        <v>1.996</v>
       </c>
       <c r="W13" t="n">
-        <v>1.9896</v>
+        <v>1.984</v>
       </c>
       <c r="X13" t="n">
-        <v>3.976</v>
+        <v>3.98</v>
       </c>
       <c r="Y13" t="n">
-        <v>2.924</v>
+        <v>2.53</v>
       </c>
       <c r="Z13" t="n">
         <v>1.339</v>
       </c>
       <c r="AA13" t="n">
-        <v>1.09</v>
+        <v>0.9025</v>
       </c>
       <c r="AB13" t="n">
-        <v>1.245</v>
+        <v>1.0575</v>
       </c>
       <c r="AC13" t="n">
         <v>0.11</v>
       </c>
       <c r="AD13" t="n">
-        <v>1.406</v>
+        <v>1.1875</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.375</v>
+        <v>0.315</v>
       </c>
       <c r="AF13" t="n">
-        <v>1.2205</v>
+        <v>0.9845</v>
       </c>
       <c r="AG13" t="n">
         <v>0.63</v>
@@ -2866,28 +2866,28 @@
         <v>0.05</v>
       </c>
       <c r="AJ13" t="n">
-        <v>1.9864</v>
+        <v>1.996</v>
       </c>
       <c r="AK13" t="n">
-        <v>1.9896</v>
+        <v>1.984</v>
       </c>
       <c r="AL13" t="n">
-        <v>3.976</v>
+        <v>3.98</v>
       </c>
       <c r="AM13" t="n">
-        <v>3.554</v>
+        <v>3.16</v>
       </c>
       <c r="AN13" t="n">
         <v>1.004</v>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>1704-20-32-Tube</t>
+          <t>1704-20-24-Tube</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -32</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -24</t>
         </is>
       </c>
       <c r="AQ13" t="inlineStr">
@@ -2902,22 +2902,22 @@
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -32 (O 2.812)</t>
+          <t>SAE code 61 flange head -24 (O 2.375)</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>3.976</t>
+          <t>3.980</t>
         </is>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>3.504</t>
+          <t>3.110</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>1.990</t>
+          <t>1.984</t>
         </is>
       </c>
       <c r="AW13" t="inlineStr">
@@ -2932,49 +2932,49 @@
       </c>
       <c r="AY13" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-32 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-24 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-20-32: L1 3.976 L2 3.504 AF 1.688 JT 0.531 GT 0.958 AFL 2.812 EFL 0.375 BFL 2.49 DFL 2.441 FFL 0.63 DRILLFL 1.004 TOD 1.339 EXT 2.487 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1704-20-24: L1 3.98 L2 3.11 AF 1.6875 JT 0.531 GT 0.958 AFL 2.375 EFL 0.315 BFL 2.12 DFL 1.969 FFL 0.63 DRILLFL 1.004 TOD 1.339 EXT 2.480 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA13" t="inlineStr">
         <is>
-          <t>1704-20-32-Tube</t>
+          <t>1704-20-24-Tube</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1704-24-16-Tube</t>
+          <t>1704-20-32-Tube</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.713041</v>
+        <v>1.488952</v>
       </c>
       <c r="C14" t="n">
-        <v>1.154701</v>
+        <v>0.974567</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9375</v>
+        <v>0.8125</v>
       </c>
       <c r="E14" t="n">
         <v>0.125</v>
       </c>
       <c r="F14" t="n">
-        <v>0.5454</v>
+        <v>0.4316</v>
       </c>
       <c r="G14" t="n">
-        <v>0.8774999999999999</v>
+        <v>0.753</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1298</v>
+        <v>0.1288</v>
       </c>
       <c r="I14" t="n">
-        <v>0.2482</v>
+        <v>0.2382</v>
       </c>
       <c r="J14" t="n">
         <v>60</v>
@@ -2983,13 +2983,13 @@
         <v>37</v>
       </c>
       <c r="L14" t="n">
-        <v>1.875</v>
+        <v>1.625</v>
       </c>
       <c r="M14" t="n">
         <v>0.08333</v>
       </c>
       <c r="N14" t="n">
-        <v>0.9234</v>
+        <v>0.7986</v>
       </c>
       <c r="O14" t="n">
         <v>0.04511</v>
@@ -3001,82 +3001,82 @@
         <v>0.08333</v>
       </c>
       <c r="R14" t="n">
-        <v>2</v>
+        <v>1.688</v>
       </c>
       <c r="S14" t="n">
-        <v>1.083041</v>
+        <v>0.957952</v>
       </c>
       <c r="T14" t="n">
-        <v>0.63</v>
+        <v>0.531</v>
       </c>
       <c r="U14" t="n">
-        <v>1.083041</v>
+        <v>0.957952</v>
       </c>
       <c r="V14" t="n">
-        <v>2.2006</v>
+        <v>1.9864</v>
       </c>
       <c r="W14" t="n">
-        <v>1.8384</v>
+        <v>1.9896</v>
       </c>
       <c r="X14" t="n">
-        <v>4.039</v>
+        <v>3.976</v>
       </c>
       <c r="Y14" t="n">
-        <v>2.348</v>
+        <v>2.924</v>
       </c>
       <c r="Z14" t="n">
-        <v>1.043</v>
+        <v>1.339</v>
       </c>
       <c r="AA14" t="n">
-        <v>0.625</v>
+        <v>1.09</v>
       </c>
       <c r="AB14" t="n">
-        <v>0.78</v>
+        <v>1.245</v>
       </c>
       <c r="AC14" t="n">
         <v>0.11</v>
       </c>
       <c r="AD14" t="n">
-        <v>0.875</v>
+        <v>1.406</v>
       </c>
       <c r="AE14" t="n">
-        <v>0.315</v>
+        <v>0.375</v>
       </c>
       <c r="AF14" t="n">
-        <v>0.748</v>
+        <v>1.2205</v>
       </c>
       <c r="AG14" t="n">
-        <v>0.551</v>
+        <v>0.63</v>
       </c>
       <c r="AH14" t="n">
-        <v>0.501</v>
+        <v>0.58</v>
       </c>
       <c r="AI14" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ14" t="n">
-        <v>2.2006</v>
+        <v>1.9864</v>
       </c>
       <c r="AK14" t="n">
-        <v>1.8384</v>
+        <v>1.9896</v>
       </c>
       <c r="AL14" t="n">
-        <v>4.039</v>
+        <v>3.976</v>
       </c>
       <c r="AM14" t="n">
-        <v>2.899</v>
+        <v>3.554</v>
       </c>
       <c r="AN14" t="n">
-        <v>0.75</v>
+        <v>1.004</v>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>1704-24-16-Tube</t>
+          <t>1704-20-32-Tube</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 61 flange -16</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 61 flange -32</t>
         </is>
       </c>
       <c r="AQ14" t="inlineStr">
@@ -3086,32 +3086,32 @@
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>1 7/8-12 (male JIC 37 deg)</t>
+          <t>1 5/8-12 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -16 (O 1.75)</t>
+          <t>SAE code 61 flange head -32 (O 2.812)</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>4.039</t>
+          <t>3.976</t>
         </is>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>2.849</t>
+          <t>3.504</t>
         </is>
       </c>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>1.838</t>
+          <t>1.990</t>
         </is>
       </c>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>1.043</t>
+          <t>1.339</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr">
@@ -3121,24 +3121,24 @@
       </c>
       <c r="AY14" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-24-16 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-20-32 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-24-16: L1 4.039 L2 2.849 AF 2.0 JT 0.63 GT 1.083 AFL 1.75 EFL 0.315 BFL 1.56 DFL 1.496 FFL 0.551 DRILLFL 0.75 TOD 1.043 EXT 2.298 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1704-20-32: L1 3.976 L2 3.504 AF 1.688 JT 0.531 GT 0.958 AFL 2.812 EFL 0.375 BFL 2.49 DFL 2.441 FFL 0.63 DRILLFL 1.004 TOD 1.339 EXT 2.487 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA14" t="inlineStr">
         <is>
-          <t>1704-24-16-Tube</t>
+          <t>1704-20-32-Tube</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1704-24-20-Tube</t>
+          <t>1704-24-16-Tube</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -3202,37 +3202,37 @@
         <v>1.083041</v>
       </c>
       <c r="V15" t="n">
-        <v>2.0744</v>
+        <v>2.2006</v>
       </c>
       <c r="W15" t="n">
-        <v>1.4456</v>
+        <v>1.8384</v>
       </c>
       <c r="X15" t="n">
-        <v>3.52</v>
+        <v>4.039</v>
       </c>
       <c r="Y15" t="n">
-        <v>1.999</v>
+        <v>2.348</v>
       </c>
       <c r="Z15" t="n">
-        <v>1.339</v>
+        <v>1.043</v>
       </c>
       <c r="AA15" t="n">
-        <v>0.72</v>
+        <v>0.625</v>
       </c>
       <c r="AB15" t="n">
-        <v>0.875</v>
+        <v>0.78</v>
       </c>
       <c r="AC15" t="n">
         <v>0.11</v>
       </c>
       <c r="AD15" t="n">
-        <v>1</v>
+        <v>0.875</v>
       </c>
       <c r="AE15" t="n">
         <v>0.315</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.8465</v>
+        <v>0.748</v>
       </c>
       <c r="AG15" t="n">
         <v>0.551</v>
@@ -3244,28 +3244,28 @@
         <v>0.05</v>
       </c>
       <c r="AJ15" t="n">
-        <v>2.0744</v>
+        <v>2.2006</v>
       </c>
       <c r="AK15" t="n">
-        <v>1.4456</v>
+        <v>1.8384</v>
       </c>
       <c r="AL15" t="n">
-        <v>3.52</v>
+        <v>4.039</v>
       </c>
       <c r="AM15" t="n">
-        <v>2.55</v>
+        <v>2.899</v>
       </c>
       <c r="AN15" t="n">
-        <v>1.08</v>
+        <v>0.75</v>
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>1704-24-20-Tube</t>
+          <t>1704-24-16-Tube</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 61 flange -20</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 61 flange -16</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
@@ -3280,27 +3280,27 @@
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -20 (O 2)</t>
+          <t>SAE code 61 flange head -16 (O 1.75)</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>3.520</t>
+          <t>4.039</t>
         </is>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.849</t>
         </is>
       </c>
       <c r="AV15" t="inlineStr">
         <is>
-          <t>1.446</t>
+          <t>1.838</t>
         </is>
       </c>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>1.339</t>
+          <t>1.043</t>
         </is>
       </c>
       <c r="AX15" t="inlineStr">
@@ -3310,24 +3310,24 @@
       </c>
       <c r="AY15" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: HEXL TUBEOD RB HUBD HUBL] [AIRWAY s115 1701-61-24-20: M1 L1 CHEX O D] Brennan CAD record 1704-24-20 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-24-16 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ15" t="inlineStr">
         <is>
-          <t>Brennan record 1704-24-20: L1 4.21 L2 3.03 AF 2.0 JT 0.63 GT 1.083 AFL 2.0 EFL 0.315 BFL 1.75 DFL 1.693 FFL 0.551 DRILLFL 1.004 TOD 1.339 EXT 2.479 (codes: README s2). Air-Way s115 1701-61-24-20 first for M1 / L1 / CHEX / O / D (user 2026-10-20 rule; settles the Air-Way-vs-Brennan differences: Brennan L1 4.21 / L2 3.03 / A/F 2.0 / AFL 2.0 / DRILLFL 1.004) Air-Way and Brennan differ beyond rounding (M3 / N4 / D) - built to Air-Way</t>
+          <t xml:space="preserve">Brennan record 1704-24-16: L1 4.039 L2 2.849 AF 2.0 JT 0.63 GT 1.083 AFL 1.75 EFL 0.315 BFL 1.56 DFL 1.496 FFL 0.551 DRILLFL 0.75 TOD 1.043 EXT 2.298 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA15" t="inlineStr">
         <is>
-          <t>1704-24-20-Tube</t>
+          <t>1704-24-16-Tube</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1704-24-24-Tube</t>
+          <t>1704-24-20-Tube</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -3391,70 +3391,70 @@
         <v>1.083041</v>
       </c>
       <c r="V16" t="n">
-        <v>2.1044</v>
+        <v>2.0744</v>
       </c>
       <c r="W16" t="n">
-        <v>1.5656</v>
+        <v>1.4456</v>
       </c>
       <c r="X16" t="n">
-        <v>3.67</v>
+        <v>3.52</v>
       </c>
       <c r="Y16" t="n">
-        <v>2.17</v>
+        <v>1.999</v>
       </c>
       <c r="Z16" t="n">
-        <v>1.575</v>
+        <v>1.339</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.9025</v>
+        <v>0.72</v>
       </c>
       <c r="AB16" t="n">
-        <v>1.0575</v>
+        <v>0.875</v>
       </c>
       <c r="AC16" t="n">
         <v>0.11</v>
       </c>
       <c r="AD16" t="n">
-        <v>1.19</v>
+        <v>1</v>
       </c>
       <c r="AE16" t="n">
         <v>0.315</v>
       </c>
       <c r="AF16" t="n">
-        <v>0.9845</v>
+        <v>0.8465</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.63</v>
+        <v>0.551</v>
       </c>
       <c r="AH16" t="n">
-        <v>0.58</v>
+        <v>0.501</v>
       </c>
       <c r="AI16" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ16" t="n">
-        <v>2.1044</v>
+        <v>2.0744</v>
       </c>
       <c r="AK16" t="n">
-        <v>1.5656</v>
+        <v>1.4456</v>
       </c>
       <c r="AL16" t="n">
-        <v>3.67</v>
+        <v>3.52</v>
       </c>
       <c r="AM16" t="n">
-        <v>2.8</v>
+        <v>2.55</v>
       </c>
       <c r="AN16" t="n">
-        <v>1.31</v>
+        <v>1.08</v>
       </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>1704-24-24-Tube</t>
+          <t>1704-24-20-Tube</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 61 flange -24</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 61 flange -20</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
@@ -3469,27 +3469,27 @@
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -24 (O 2.38)</t>
+          <t>SAE code 61 flange head -20 (O 2)</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>3.670</t>
+          <t>3.520</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>2.750</t>
+          <t>2.500</t>
         </is>
       </c>
       <c r="AV16" t="inlineStr">
         <is>
-          <t>1.566</t>
+          <t>1.446</t>
         </is>
       </c>
       <c r="AW16" t="inlineStr">
         <is>
-          <t>1.575</t>
+          <t>1.339</t>
         </is>
       </c>
       <c r="AX16" t="inlineStr">
@@ -3499,24 +3499,24 @@
       </c>
       <c r="AY16" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: HEXL TUBEOD RB HUBD HUBL] [AIRWAY s115 1701-61-24-24: M1 L1 CHEX O D] Brennan CAD record 1704-24-24 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: HEXL TUBEOD RB HUBD HUBL] [AIRWAY s115 1701-61-24-20: M1 L1 CHEX O D] Brennan CAD record 1704-24-20 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ16" t="inlineStr">
         <is>
-          <t>Brennan record 1704-24-24: L1 4.57 L2 3.66 AF 2.0 JT 0.63 GT 1.083 AFL 2.375 EFL 0.315 BFL 2.12 DFL 1.969 FFL 0.63 DRILLFL 1.23 TOD 1.575 EXT 2.857 (codes: README s2). Air-Way s115 1701-61-24-24 first for M1 / L1 / CHEX / O / D (user 2026-10-20 rule; settles the Air-Way-vs-Brennan differences: Brennan L1 4.57 / L2 3.66 / A/F 2.0 / AFL 2.375 / DRILLFL 1.23) Air-Way and Brennan differ beyond rounding (M3 / N4 / D) - built to Air-Way</t>
+          <t>Brennan record 1704-24-20: L1 4.21 L2 3.03 AF 2.0 JT 0.63 GT 1.083 AFL 2.0 EFL 0.315 BFL 1.75 DFL 1.693 FFL 0.551 DRILLFL 1.004 TOD 1.339 EXT 2.479 (codes: README s2). Air-Way s115 1701-61-24-20 first for M1 / L1 / CHEX / O / D (user 2026-10-20 rule; settles the Air-Way-vs-Brennan differences: Brennan L1 4.21 / L2 3.03 / A/F 2.0 / AFL 2.0 / DRILLFL 1.004) Air-Way and Brennan differ beyond rounding (M3 / N4 / D) - built to Air-Way</t>
         </is>
       </c>
       <c r="BA16" t="inlineStr">
         <is>
-          <t>1704-24-24-Tube</t>
+          <t>1704-24-20-Tube</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1704-24-32-Tube</t>
+          <t>1704-24-24-Tube</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3580,37 +3580,37 @@
         <v>1.083041</v>
       </c>
       <c r="V17" t="n">
-        <v>2.2844</v>
+        <v>2.1044</v>
       </c>
       <c r="W17" t="n">
-        <v>2.2856</v>
+        <v>1.5656</v>
       </c>
       <c r="X17" t="n">
-        <v>4.57</v>
+        <v>3.67</v>
       </c>
       <c r="Y17" t="n">
-        <v>3.28</v>
+        <v>2.17</v>
       </c>
       <c r="Z17" t="n">
         <v>1.575</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.09</v>
+        <v>0.9025</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.245</v>
+        <v>1.0575</v>
       </c>
       <c r="AC17" t="n">
         <v>0.11</v>
       </c>
       <c r="AD17" t="n">
-        <v>1.406</v>
+        <v>1.19</v>
       </c>
       <c r="AE17" t="n">
-        <v>0.375</v>
+        <v>0.315</v>
       </c>
       <c r="AF17" t="n">
-        <v>1.2205</v>
+        <v>0.9845</v>
       </c>
       <c r="AG17" t="n">
         <v>0.63</v>
@@ -3622,28 +3622,28 @@
         <v>0.05</v>
       </c>
       <c r="AJ17" t="n">
-        <v>2.2844</v>
+        <v>2.1044</v>
       </c>
       <c r="AK17" t="n">
-        <v>2.2856</v>
+        <v>1.5656</v>
       </c>
       <c r="AL17" t="n">
-        <v>4.57</v>
+        <v>3.67</v>
       </c>
       <c r="AM17" t="n">
-        <v>3.91</v>
+        <v>2.8</v>
       </c>
       <c r="AN17" t="n">
-        <v>1.23</v>
+        <v>1.31</v>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>1704-24-32-Tube</t>
+          <t>1704-24-24-Tube</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 61 flange -32</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 61 flange -24</t>
         </is>
       </c>
       <c r="AQ17" t="inlineStr">
@@ -3658,22 +3658,22 @@
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -32 (O 2.812)</t>
+          <t>SAE code 61 flange head -24 (O 2.38)</t>
         </is>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>4.570</t>
+          <t>3.670</t>
         </is>
       </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>3.860</t>
+          <t>2.750</t>
         </is>
       </c>
       <c r="AV17" t="inlineStr">
         <is>
-          <t>2.286</t>
+          <t>1.566</t>
         </is>
       </c>
       <c r="AW17" t="inlineStr">
@@ -3688,49 +3688,49 @@
       </c>
       <c r="AY17" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-24-32 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: HEXL TUBEOD RB HUBD HUBL] [AIRWAY s115 1701-61-24-24: M1 L1 CHEX O D] Brennan CAD record 1704-24-24 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-24-32: L1 4.57 L2 3.86 AF 2.0 JT 0.63 GT 1.083 AFL 2.812 EFL 0.375 BFL 2.49 DFL 2.441 FFL 0.63 DRILLFL 1.23 TOD 1.575 EXT 2.857 (codes: README s2). </t>
+          <t>Brennan record 1704-24-24: L1 4.57 L2 3.66 AF 2.0 JT 0.63 GT 1.083 AFL 2.375 EFL 0.315 BFL 2.12 DFL 1.969 FFL 0.63 DRILLFL 1.23 TOD 1.575 EXT 2.857 (codes: README s2). Air-Way s115 1701-61-24-24 first for M1 / L1 / CHEX / O / D (user 2026-10-20 rule; settles the Air-Way-vs-Brennan differences: Brennan L1 4.57 / L2 3.66 / A/F 2.0 / AFL 2.375 / DRILLFL 1.23) Air-Way and Brennan differ beyond rounding (M3 / N4 / D) - built to Air-Way</t>
         </is>
       </c>
       <c r="BA17" t="inlineStr">
         <is>
-          <t>1704-24-32-Tube</t>
+          <t>1704-24-24-Tube</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1704-32-24-Tube</t>
+          <t>1704-24-32-Tube</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1.963041</v>
+        <v>1.713041</v>
       </c>
       <c r="C18" t="n">
-        <v>1.587713</v>
+        <v>1.154701</v>
       </c>
       <c r="D18" t="n">
-        <v>1.25</v>
+        <v>0.9375</v>
       </c>
       <c r="E18" t="n">
         <v>0.125</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7124</v>
+        <v>0.5454</v>
       </c>
       <c r="G18" t="n">
-        <v>1.19</v>
+        <v>0.8774999999999999</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1292</v>
+        <v>0.1298</v>
       </c>
       <c r="I18" t="n">
-        <v>0.3318</v>
+        <v>0.2482</v>
       </c>
       <c r="J18" t="n">
         <v>60</v>
@@ -3739,13 +3739,13 @@
         <v>37</v>
       </c>
       <c r="L18" t="n">
-        <v>2.5</v>
+        <v>1.875</v>
       </c>
       <c r="M18" t="n">
         <v>0.08333</v>
       </c>
       <c r="N18" t="n">
-        <v>1.1734</v>
+        <v>0.9234</v>
       </c>
       <c r="O18" t="n">
         <v>0.04511</v>
@@ -3757,49 +3757,49 @@
         <v>0.08333</v>
       </c>
       <c r="R18" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="S18" t="n">
-        <v>1.333041</v>
+        <v>1.083041</v>
       </c>
       <c r="T18" t="n">
         <v>0.63</v>
       </c>
       <c r="U18" t="n">
-        <v>1.333041</v>
+        <v>1.083041</v>
       </c>
       <c r="V18" t="n">
-        <v>2.616</v>
+        <v>2.2844</v>
       </c>
       <c r="W18" t="n">
-        <v>2.424</v>
+        <v>2.2856</v>
       </c>
       <c r="X18" t="n">
-        <v>5.04</v>
+        <v>4.57</v>
       </c>
       <c r="Y18" t="n">
-        <v>3.08</v>
+        <v>3.28</v>
       </c>
       <c r="Z18" t="n">
         <v>1.575</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.9025</v>
+        <v>1.09</v>
       </c>
       <c r="AB18" t="n">
-        <v>1.0575</v>
+        <v>1.245</v>
       </c>
       <c r="AC18" t="n">
         <v>0.11</v>
       </c>
       <c r="AD18" t="n">
-        <v>1.1875</v>
+        <v>1.406</v>
       </c>
       <c r="AE18" t="n">
-        <v>0.315</v>
+        <v>0.375</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.9845</v>
+        <v>1.2205</v>
       </c>
       <c r="AG18" t="n">
         <v>0.63</v>
@@ -3811,28 +3811,28 @@
         <v>0.05</v>
       </c>
       <c r="AJ18" t="n">
-        <v>2.616</v>
+        <v>2.2844</v>
       </c>
       <c r="AK18" t="n">
-        <v>2.424</v>
+        <v>2.2856</v>
       </c>
       <c r="AL18" t="n">
-        <v>5.04</v>
+        <v>4.57</v>
       </c>
       <c r="AM18" t="n">
-        <v>3.71</v>
+        <v>3.91</v>
       </c>
       <c r="AN18" t="n">
         <v>1.23</v>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>1704-32-24-Tube</t>
+          <t>1704-24-32-Tube</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -32 x code 61 flange -24</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 61 flange -32</t>
         </is>
       </c>
       <c r="AQ18" t="inlineStr">
@@ -3842,27 +3842,27 @@
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>2 1/2-12 (male JIC 37 deg)</t>
+          <t>1 7/8-12 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -24 (O 2.375)</t>
+          <t>SAE code 61 flange head -32 (O 2.812)</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>5.040</t>
+          <t>4.570</t>
         </is>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>3.660</t>
+          <t>3.860</t>
         </is>
       </c>
       <c r="AV18" t="inlineStr">
         <is>
-          <t>2.424</t>
+          <t>2.286</t>
         </is>
       </c>
       <c r="AW18" t="inlineStr">
@@ -3877,24 +3877,24 @@
       </c>
       <c r="AY18" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-32-24 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-24-32 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-32-24: L1 5.04 L2 3.66 AF 2.75 JT 0.63 GT 1.333 AFL 2.375 EFL 0.315 BFL 2.12 DFL 1.969 FFL 0.63 DRILLFL 1.23 TOD 1.575 EXT 3.030 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1704-24-32: L1 4.57 L2 3.86 AF 2.0 JT 0.63 GT 1.083 AFL 2.812 EFL 0.375 BFL 2.49 DFL 2.441 FFL 0.63 DRILLFL 1.23 TOD 1.575 EXT 2.857 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA18" t="inlineStr">
         <is>
-          <t>1704-32-24-Tube</t>
+          <t>1704-24-32-Tube</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1704-32-32-Tube</t>
+          <t>1704-32-24-Tube</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3958,37 +3958,37 @@
         <v>1.333041</v>
       </c>
       <c r="V19" t="n">
-        <v>2.7284</v>
+        <v>2.616</v>
       </c>
       <c r="W19" t="n">
-        <v>3.0616</v>
+        <v>2.424</v>
       </c>
       <c r="X19" t="n">
-        <v>5.79</v>
+        <v>5.04</v>
       </c>
       <c r="Y19" t="n">
-        <v>4.26</v>
+        <v>3.08</v>
       </c>
       <c r="Z19" t="n">
-        <v>2.087</v>
+        <v>1.575</v>
       </c>
       <c r="AA19" t="n">
-        <v>1.09</v>
+        <v>0.9025</v>
       </c>
       <c r="AB19" t="n">
-        <v>1.245</v>
+        <v>1.0575</v>
       </c>
       <c r="AC19" t="n">
         <v>0.11</v>
       </c>
       <c r="AD19" t="n">
-        <v>1.406</v>
+        <v>1.1875</v>
       </c>
       <c r="AE19" t="n">
-        <v>0.375</v>
+        <v>0.315</v>
       </c>
       <c r="AF19" t="n">
-        <v>1.2205</v>
+        <v>0.9845</v>
       </c>
       <c r="AG19" t="n">
         <v>0.63</v>
@@ -4000,28 +4000,28 @@
         <v>0.05</v>
       </c>
       <c r="AJ19" t="n">
-        <v>2.7284</v>
+        <v>2.616</v>
       </c>
       <c r="AK19" t="n">
-        <v>3.0616</v>
+        <v>2.424</v>
       </c>
       <c r="AL19" t="n">
-        <v>5.79</v>
+        <v>5.04</v>
       </c>
       <c r="AM19" t="n">
-        <v>4.89</v>
+        <v>3.71</v>
       </c>
       <c r="AN19" t="n">
-        <v>1.693</v>
+        <v>1.23</v>
       </c>
       <c r="AO19" t="inlineStr">
         <is>
-          <t>1704-32-32-Tube</t>
+          <t>1704-32-24-Tube</t>
         </is>
       </c>
       <c r="AP19" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -32 x code 61 flange -32</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -32 x code 61 flange -24</t>
         </is>
       </c>
       <c r="AQ19" t="inlineStr">
@@ -4036,27 +4036,27 @@
       </c>
       <c r="AS19" t="inlineStr">
         <is>
-          <t>SAE code 61 flange head -32 (O 2.812)</t>
+          <t>SAE code 61 flange head -24 (O 2.375)</t>
         </is>
       </c>
       <c r="AT19" t="inlineStr">
         <is>
-          <t>5.790</t>
+          <t>5.040</t>
         </is>
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>4.840</t>
+          <t>3.660</t>
         </is>
       </c>
       <c r="AV19" t="inlineStr">
         <is>
-          <t>3.062</t>
+          <t>2.424</t>
         </is>
       </c>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>2.087</t>
+          <t>1.575</t>
         </is>
       </c>
       <c r="AX19" t="inlineStr">
@@ -4066,49 +4066,49 @@
       </c>
       <c r="AY19" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-32-32 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-32-24 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1704-32-32: L1 5.79 L2 4.84 AF 2.75 JT 0.63 GT 1.333 AFL 2.812 EFL 0.375 BFL 2.49 DFL 2.441 FFL 0.63 DRILLFL 1.693 TOD 2.087 EXT 3.827 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1704-32-24: L1 5.04 L2 3.66 AF 2.75 JT 0.63 GT 1.333 AFL 2.375 EFL 0.315 BFL 2.12 DFL 1.969 FFL 0.63 DRILLFL 1.23 TOD 1.575 EXT 3.030 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA19" t="inlineStr">
         <is>
-          <t>1704-32-32-Tube</t>
+          <t>1704-32-24-Tube</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1804-08-08-Tube</t>
+          <t>1704-32-32-Tube</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.050969</v>
+        <v>1.963041</v>
       </c>
       <c r="C20" t="n">
-        <v>0.505181</v>
+        <v>1.587713</v>
       </c>
       <c r="D20" t="n">
-        <v>0.375</v>
+        <v>1.25</v>
       </c>
       <c r="E20" t="n">
-        <v>0.094</v>
+        <v>0.125</v>
       </c>
       <c r="F20" t="n">
-        <v>0.2837</v>
+        <v>0.7124</v>
       </c>
       <c r="G20" t="n">
-        <v>0.3295</v>
+        <v>1.19</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0984</v>
+        <v>0.1292</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1546</v>
+        <v>0.3318</v>
       </c>
       <c r="J20" t="n">
         <v>60</v>
@@ -4117,100 +4117,100 @@
         <v>37</v>
       </c>
       <c r="L20" t="n">
-        <v>0.75</v>
+        <v>2.5</v>
       </c>
       <c r="M20" t="n">
-        <v>0.0625</v>
+        <v>0.08333</v>
       </c>
       <c r="N20" t="n">
-        <v>0.5367</v>
+        <v>1.1734</v>
       </c>
       <c r="O20" t="n">
-        <v>0.03383</v>
+        <v>0.04511</v>
       </c>
       <c r="P20" t="n">
-        <v>0.01562</v>
+        <v>0.02083</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.0625</v>
+        <v>0.08333</v>
       </c>
       <c r="R20" t="n">
-        <v>0.875</v>
+        <v>2.75</v>
       </c>
       <c r="S20" t="n">
-        <v>0.656969</v>
+        <v>1.333041</v>
       </c>
       <c r="T20" t="n">
-        <v>0.394</v>
+        <v>0.63</v>
       </c>
       <c r="U20" t="n">
-        <v>0.656969</v>
+        <v>1.333041</v>
       </c>
       <c r="V20" t="n">
-        <v>1.3048</v>
+        <v>2.7284</v>
       </c>
       <c r="W20" t="n">
-        <v>1.0152</v>
+        <v>3.0616</v>
       </c>
       <c r="X20" t="n">
-        <v>2.32</v>
+        <v>5.79</v>
       </c>
       <c r="Y20" t="n">
-        <v>1.349</v>
+        <v>4.26</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.618</v>
+        <v>2.087</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.345</v>
+        <v>1.09</v>
       </c>
       <c r="AB20" t="n">
-        <v>0.5</v>
+        <v>1.245</v>
       </c>
       <c r="AC20" t="n">
         <v>0.11</v>
       </c>
       <c r="AD20" t="n">
-        <v>0.625</v>
+        <v>1.406</v>
       </c>
       <c r="AE20" t="n">
-        <v>0.305</v>
+        <v>0.375</v>
       </c>
       <c r="AF20" t="n">
-        <v>0.4725</v>
+        <v>1.2205</v>
       </c>
       <c r="AG20" t="n">
-        <v>0.551</v>
+        <v>0.63</v>
       </c>
       <c r="AH20" t="n">
-        <v>0.501</v>
+        <v>0.58</v>
       </c>
       <c r="AI20" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ20" t="n">
-        <v>1.3048</v>
+        <v>2.7284</v>
       </c>
       <c r="AK20" t="n">
-        <v>1.0152</v>
+        <v>3.0616</v>
       </c>
       <c r="AL20" t="n">
-        <v>2.32</v>
+        <v>5.79</v>
       </c>
       <c r="AM20" t="n">
-        <v>1.9</v>
+        <v>4.89</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.374</v>
+        <v>1.693</v>
       </c>
       <c r="AO20" t="inlineStr">
         <is>
-          <t>1804-08-08-Tube</t>
+          <t>1704-32-32-Tube</t>
         </is>
       </c>
       <c r="AP20" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -08 x code 62 flange -08</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -32 x code 61 flange -32</t>
         </is>
       </c>
       <c r="AQ20" t="inlineStr">
@@ -4220,32 +4220,32 @@
       </c>
       <c r="AR20" t="inlineStr">
         <is>
-          <t>3/4-16 (male JIC 37 deg)</t>
+          <t>2 1/2-12 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS20" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -08 (O 1.25)</t>
+          <t>SAE code 61 flange head -32 (O 2.812)</t>
         </is>
       </c>
       <c r="AT20" t="inlineStr">
         <is>
-          <t>2.320</t>
+          <t>5.790</t>
         </is>
       </c>
       <c r="AU20" t="inlineStr">
         <is>
-          <t>1.850</t>
+          <t>4.840</t>
         </is>
       </c>
       <c r="AV20" t="inlineStr">
         <is>
-          <t>1.015</t>
+          <t>3.062</t>
         </is>
       </c>
       <c r="AW20" t="inlineStr">
         <is>
-          <t>0.618</t>
+          <t>2.087</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
@@ -4255,49 +4255,49 @@
       </c>
       <c r="AY20" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-08-08 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head: thickness and face O-ring groove by flange size measured on the Brennan 1800-08-08 / 1824-08 / 1804-08-08-FG STEPs (wave-1 FLANGE62, flange62.py; single manufacturer - SAE J518 / ISO 6162-2 not in the repo), head OD = the row (must equal the measured 1.250 at -08); edge chamfers not modelled; -08 only (no STEP with a -12..-32 code 62 head); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1704-32-32 decoded on BRENNAN_1704-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p005-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 61 flange head (FLG61_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 61 flange head: head OD = Air-Way O, head thickness and face O-ring groove (inner/outer dia, depth 0.11) measured on the Brennan 1700-08/-12/-16/-20/-24/-32 STEPs by flange size (single source - SAE J518 not available); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-08-08: L1 2.32 L2 1.85 AF 0.875 JT 0.394 GT 0.657 AFL 1.25 EFL 0.305 BFL 1.0 DFL 0.945 FFL 0.551 DRILLFL 0.374 TOD 0.618 EXT 1.269 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1704-32-32: L1 5.79 L2 4.84 AF 2.75 JT 0.63 GT 1.333 AFL 2.812 EFL 0.375 BFL 2.49 DFL 2.441 FFL 0.63 DRILLFL 1.693 TOD 2.087 EXT 3.827 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA20" t="inlineStr">
         <is>
-          <t>1804-08-08-Tube</t>
+          <t>1704-32-32-Tube</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1804-12-12-Tube</t>
+          <t>1804-08-08-Tube</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.257997</v>
+        <v>1.050969</v>
       </c>
       <c r="C21" t="n">
-        <v>0.649519</v>
+        <v>0.505181</v>
       </c>
       <c r="D21" t="n">
-        <v>0.53125</v>
+        <v>0.375</v>
       </c>
       <c r="E21" t="n">
-        <v>0.125</v>
+        <v>0.094</v>
       </c>
       <c r="F21" t="n">
-        <v>0.3895</v>
+        <v>0.2837</v>
       </c>
       <c r="G21" t="n">
-        <v>0.4715</v>
+        <v>0.3295</v>
       </c>
       <c r="H21" t="n">
-        <v>0.1299</v>
+        <v>0.0984</v>
       </c>
       <c r="I21" t="n">
-        <v>0.1851</v>
+        <v>0.1546</v>
       </c>
       <c r="J21" t="n">
         <v>60</v>
@@ -4306,100 +4306,100 @@
         <v>37</v>
       </c>
       <c r="L21" t="n">
-        <v>1.0625</v>
+        <v>0.75</v>
       </c>
       <c r="M21" t="n">
-        <v>0.08333</v>
+        <v>0.0625</v>
       </c>
       <c r="N21" t="n">
-        <v>0.7045</v>
+        <v>0.5367</v>
       </c>
       <c r="O21" t="n">
-        <v>0.04511</v>
+        <v>0.03383</v>
       </c>
       <c r="P21" t="n">
-        <v>0.02083</v>
+        <v>0.01562</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.08333</v>
+        <v>0.0625</v>
       </c>
       <c r="R21" t="n">
-        <v>1.125</v>
+        <v>0.875</v>
       </c>
       <c r="S21" t="n">
-        <v>0.863997</v>
+        <v>0.656969</v>
       </c>
       <c r="T21" t="n">
         <v>0.394</v>
       </c>
       <c r="U21" t="n">
-        <v>0.863997</v>
+        <v>0.656969</v>
       </c>
       <c r="V21" t="n">
-        <v>1.5732</v>
+        <v>1.3048</v>
       </c>
       <c r="W21" t="n">
-        <v>1.2568</v>
+        <v>1.0152</v>
       </c>
       <c r="X21" t="n">
-        <v>2.83</v>
+        <v>2.32</v>
       </c>
       <c r="Y21" t="n">
-        <v>1.621</v>
+        <v>1.349</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.8</v>
+        <v>0.618</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.47</v>
+        <v>0.345</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.625</v>
+        <v>0.5</v>
       </c>
       <c r="AC21" t="n">
         <v>0.11</v>
       </c>
       <c r="AD21" t="n">
-        <v>0.8125</v>
+        <v>0.625</v>
       </c>
       <c r="AE21" t="n">
-        <v>0.345</v>
+        <v>0.305</v>
       </c>
       <c r="AF21" t="n">
-        <v>0.63</v>
+        <v>0.4725</v>
       </c>
       <c r="AG21" t="n">
-        <v>0.709</v>
+        <v>0.551</v>
       </c>
       <c r="AH21" t="n">
-        <v>0.659</v>
+        <v>0.501</v>
       </c>
       <c r="AI21" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ21" t="n">
-        <v>1.5732</v>
+        <v>1.3048</v>
       </c>
       <c r="AK21" t="n">
-        <v>1.2568</v>
+        <v>1.0152</v>
       </c>
       <c r="AL21" t="n">
-        <v>2.83</v>
+        <v>2.32</v>
       </c>
       <c r="AM21" t="n">
-        <v>2.33</v>
+        <v>1.9</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.551</v>
+        <v>0.374</v>
       </c>
       <c r="AO21" t="inlineStr">
         <is>
-          <t>1804-12-12-Tube</t>
+          <t>1804-08-08-Tube</t>
         </is>
       </c>
       <c r="AP21" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -12 x code 62 flange -12</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -08 x code 62 flange -08</t>
         </is>
       </c>
       <c r="AQ21" t="inlineStr">
@@ -4409,32 +4409,32 @@
       </c>
       <c r="AR21" t="inlineStr">
         <is>
-          <t>1 1/16-12 (male JIC 37 deg)</t>
+          <t>3/4-16 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS21" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -12 (O 1.625)</t>
+          <t>SAE code 62 flange head -08 (O 1.25)</t>
         </is>
       </c>
       <c r="AT21" t="inlineStr">
         <is>
-          <t>2.830</t>
+          <t>2.320</t>
         </is>
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>2.280</t>
+          <t>1.850</t>
         </is>
       </c>
       <c r="AV21" t="inlineStr">
         <is>
-          <t>1.257</t>
+          <t>1.015</t>
         </is>
       </c>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>0.800</t>
+          <t>0.618</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr">
@@ -4444,24 +4444,24 @@
       </c>
       <c r="AY21" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-12-12 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -12: head OD / thickness / face O-ring groove measured on BRENNAN_1803-12-12.stp (= Brennan catalog 3300-62-12-12 A 1.625 / D 0.345 / H 1.250); single manufacturer - SAE J518 / ISO 6162-2 not in the repo; edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-08-08 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head: thickness and face O-ring groove by flange size measured on the Brennan 1800-08-08 / 1824-08 / 1804-08-08-FG STEPs (wave-1 FLANGE62, flange62.py; single manufacturer - SAE J518 / ISO 6162-2 not in the repo), head OD = the row (must equal the measured 1.250 at -08); edge chamfers not modelled; -08 only (no STEP with a -12..-32 code 62 head); flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-12-12: L1 2.83 L2 2.28 AF 1.125 JT 0.394 GT 0.864 AFL 1.625 EFL 0.345 BFL 1.25 DFL 1.26 FFL 0.709 DRILLFL 0.551 TOD 0.8 EXT 1.571 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-08-08: L1 2.32 L2 1.85 AF 0.875 JT 0.394 GT 0.657 AFL 1.25 EFL 0.305 BFL 1.0 DFL 0.945 FFL 0.551 DRILLFL 0.374 TOD 0.618 EXT 1.269 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA21" t="inlineStr">
         <is>
-          <t>1804-12-12-Tube</t>
+          <t>1804-08-08-Tube</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1804-12-16-Tube</t>
+          <t>1804-12-12-Tube</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -4525,70 +4525,70 @@
         <v>0.863997</v>
       </c>
       <c r="V22" t="n">
-        <v>1.5724</v>
+        <v>1.5732</v>
       </c>
       <c r="W22" t="n">
-        <v>1.2576</v>
+        <v>1.2568</v>
       </c>
       <c r="X22" t="n">
         <v>2.83</v>
       </c>
       <c r="Y22" t="n">
-        <v>1.623</v>
+        <v>1.621</v>
       </c>
       <c r="Z22" t="n">
         <v>0.8</v>
       </c>
       <c r="AA22" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB22" t="n">
         <v>0.625</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>0.78</v>
       </c>
       <c r="AC22" t="n">
         <v>0.11</v>
       </c>
       <c r="AD22" t="n">
-        <v>0.9375</v>
+        <v>0.8125</v>
       </c>
       <c r="AE22" t="n">
-        <v>0.375</v>
+        <v>0.345</v>
       </c>
       <c r="AF22" t="n">
-        <v>0.748</v>
+        <v>0.63</v>
       </c>
       <c r="AG22" t="n">
-        <v>0.827</v>
+        <v>0.709</v>
       </c>
       <c r="AH22" t="n">
-        <v>0.777</v>
+        <v>0.659</v>
       </c>
       <c r="AI22" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ22" t="n">
-        <v>1.5724</v>
+        <v>1.5732</v>
       </c>
       <c r="AK22" t="n">
-        <v>1.2576</v>
+        <v>1.2568</v>
       </c>
       <c r="AL22" t="n">
         <v>2.83</v>
       </c>
       <c r="AM22" t="n">
-        <v>2.45</v>
+        <v>2.33</v>
       </c>
       <c r="AN22" t="n">
         <v>0.551</v>
       </c>
       <c r="AO22" t="inlineStr">
         <is>
-          <t>1804-12-16-Tube</t>
+          <t>1804-12-12-Tube</t>
         </is>
       </c>
       <c r="AP22" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -12 x code 62 flange -16</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -12 x code 62 flange -12</t>
         </is>
       </c>
       <c r="AQ22" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="AS22" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -16 (O 1.875)</t>
+          <t>SAE code 62 flange head -12 (O 1.625)</t>
         </is>
       </c>
       <c r="AT22" t="inlineStr">
@@ -4613,12 +4613,12 @@
       </c>
       <c r="AU22" t="inlineStr">
         <is>
-          <t>2.400</t>
+          <t>2.280</t>
         </is>
       </c>
       <c r="AV22" t="inlineStr">
         <is>
-          <t>1.258</t>
+          <t>1.257</t>
         </is>
       </c>
       <c r="AW22" t="inlineStr">
@@ -4633,24 +4633,24 @@
       </c>
       <c r="AY22" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-12-16 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -16: head OD 1.875 / thickness 0.375 / groove OD 1.560 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.250 / depth 0.11 = the code 61 -16 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-12-12 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -12: head OD / thickness / face O-ring groove measured on BRENNAN_1803-12-12.stp (= Brennan catalog 3300-62-12-12 A 1.625 / D 0.345 / H 1.250); single manufacturer - SAE J518 / ISO 6162-2 not in the repo; edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-12-16: L1 2.83 L2 2.4 AF 1.125 JT 0.394 GT 0.864 AFL 1.875 EFL 0.375 BFL 1.56 DFL 1.496 FFL 0.827 DRILLFL 0.551 TOD 0.8 EXT 1.572 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-12-12: L1 2.83 L2 2.28 AF 1.125 JT 0.394 GT 0.864 AFL 1.625 EFL 0.345 BFL 1.25 DFL 1.26 FFL 0.709 DRILLFL 0.551 TOD 0.8 EXT 1.571 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA22" t="inlineStr">
         <is>
-          <t>1804-12-16-Tube</t>
+          <t>1804-12-12-Tube</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1804-12-20-Tube</t>
+          <t>1804-12-16-Tube</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -4723,34 +4723,34 @@
         <v>2.83</v>
       </c>
       <c r="Y23" t="n">
-        <v>1.826</v>
+        <v>1.623</v>
       </c>
       <c r="Z23" t="n">
         <v>0.8</v>
       </c>
       <c r="AA23" t="n">
-        <v>0.72</v>
+        <v>0.625</v>
       </c>
       <c r="AB23" t="n">
-        <v>0.875</v>
+        <v>0.78</v>
       </c>
       <c r="AC23" t="n">
         <v>0.11</v>
       </c>
       <c r="AD23" t="n">
-        <v>1.0625</v>
+        <v>0.9375</v>
       </c>
       <c r="AE23" t="n">
-        <v>0.405</v>
+        <v>0.375</v>
       </c>
       <c r="AF23" t="n">
-        <v>0.866</v>
+        <v>0.748</v>
       </c>
       <c r="AG23" t="n">
-        <v>0.984</v>
+        <v>0.827</v>
       </c>
       <c r="AH23" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.777</v>
       </c>
       <c r="AI23" t="n">
         <v>0.05</v>
@@ -4765,19 +4765,19 @@
         <v>2.83</v>
       </c>
       <c r="AM23" t="n">
-        <v>2.81</v>
+        <v>2.45</v>
       </c>
       <c r="AN23" t="n">
         <v>0.551</v>
       </c>
       <c r="AO23" t="inlineStr">
         <is>
-          <t>1804-12-20-Tube</t>
+          <t>1804-12-16-Tube</t>
         </is>
       </c>
       <c r="AP23" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -12 x code 62 flange -20</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -12 x code 62 flange -16</t>
         </is>
       </c>
       <c r="AQ23" t="inlineStr">
@@ -4792,7 +4792,7 @@
       </c>
       <c r="AS23" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -20 (O 2.125)</t>
+          <t>SAE code 62 flange head -16 (O 1.875)</t>
         </is>
       </c>
       <c r="AT23" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="AU23" t="inlineStr">
         <is>
-          <t>2.760</t>
+          <t>2.400</t>
         </is>
       </c>
       <c r="AV23" t="inlineStr">
@@ -4822,49 +4822,49 @@
       </c>
       <c r="AY23" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-12-20 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -20: head OD 2.125 / thickness 0.405 / groove OD 1.750 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.440 / depth 0.11 = the code 61 -20 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-12-16 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -16: head OD 1.875 / thickness 0.375 / groove OD 1.560 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.250 / depth 0.11 = the code 61 -16 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-12-20: L1 2.83 L2 2.76 AF 1.125 JT 0.394 GT 0.864 AFL 2.125 EFL 0.405 BFL 1.75 DFL 1.732 FFL 0.984 DRILLFL 0.551 TOD 0.8 EXT 1.572 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-12-16: L1 2.83 L2 2.4 AF 1.125 JT 0.394 GT 0.864 AFL 1.875 EFL 0.375 BFL 1.56 DFL 1.496 FFL 0.827 DRILLFL 0.551 TOD 0.8 EXT 1.572 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA23" t="inlineStr">
         <is>
-          <t>1804-12-20-Tube</t>
+          <t>1804-12-16-Tube</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1804-16-12-Tube</t>
+          <t>1804-12-20-Tube</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.363997</v>
+        <v>1.257997</v>
       </c>
       <c r="C24" t="n">
-        <v>0.793857</v>
+        <v>0.649519</v>
       </c>
       <c r="D24" t="n">
-        <v>0.65625</v>
+        <v>0.53125</v>
       </c>
       <c r="E24" t="n">
         <v>0.125</v>
       </c>
       <c r="F24" t="n">
-        <v>0.4365</v>
+        <v>0.3895</v>
       </c>
       <c r="G24" t="n">
-        <v>0.5965</v>
+        <v>0.4715</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1292</v>
+        <v>0.1299</v>
       </c>
       <c r="I24" t="n">
-        <v>0.1858</v>
+        <v>0.1851</v>
       </c>
       <c r="J24" t="n">
         <v>60</v>
@@ -4873,13 +4873,13 @@
         <v>37</v>
       </c>
       <c r="L24" t="n">
-        <v>1.3125</v>
+        <v>1.0625</v>
       </c>
       <c r="M24" t="n">
         <v>0.08333</v>
       </c>
       <c r="N24" t="n">
-        <v>0.7514999999999999</v>
+        <v>0.7045</v>
       </c>
       <c r="O24" t="n">
         <v>0.04511</v>
@@ -4891,82 +4891,82 @@
         <v>0.08333</v>
       </c>
       <c r="R24" t="n">
-        <v>1.375</v>
+        <v>1.125</v>
       </c>
       <c r="S24" t="n">
-        <v>0.9109969999999999</v>
+        <v>0.863997</v>
       </c>
       <c r="T24" t="n">
-        <v>0.453</v>
+        <v>0.394</v>
       </c>
       <c r="U24" t="n">
-        <v>0.9109969999999999</v>
+        <v>0.863997</v>
       </c>
       <c r="V24" t="n">
-        <v>1.6772</v>
+        <v>1.5724</v>
       </c>
       <c r="W24" t="n">
-        <v>1.2528</v>
+        <v>1.2576</v>
       </c>
       <c r="X24" t="n">
-        <v>2.93</v>
+        <v>2.83</v>
       </c>
       <c r="Y24" t="n">
-        <v>1.621</v>
+        <v>1.826</v>
       </c>
       <c r="Z24" t="n">
         <v>0.8</v>
       </c>
       <c r="AA24" t="n">
-        <v>0.47</v>
+        <v>0.72</v>
       </c>
       <c r="AB24" t="n">
-        <v>0.625</v>
+        <v>0.875</v>
       </c>
       <c r="AC24" t="n">
         <v>0.11</v>
       </c>
       <c r="AD24" t="n">
-        <v>0.8125</v>
+        <v>1.0625</v>
       </c>
       <c r="AE24" t="n">
-        <v>0.345</v>
+        <v>0.405</v>
       </c>
       <c r="AF24" t="n">
-        <v>0.63</v>
+        <v>0.866</v>
       </c>
       <c r="AG24" t="n">
-        <v>0.709</v>
+        <v>0.984</v>
       </c>
       <c r="AH24" t="n">
-        <v>0.659</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="AI24" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ24" t="n">
-        <v>1.6772</v>
+        <v>1.5724</v>
       </c>
       <c r="AK24" t="n">
-        <v>1.2528</v>
+        <v>1.2576</v>
       </c>
       <c r="AL24" t="n">
-        <v>2.93</v>
+        <v>2.83</v>
       </c>
       <c r="AM24" t="n">
-        <v>2.33</v>
+        <v>2.81</v>
       </c>
       <c r="AN24" t="n">
         <v>0.551</v>
       </c>
       <c r="AO24" t="inlineStr">
         <is>
-          <t>1804-16-12-Tube</t>
+          <t>1804-12-20-Tube</t>
         </is>
       </c>
       <c r="AP24" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -16 x code 62 flange -12</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -12 x code 62 flange -20</t>
         </is>
       </c>
       <c r="AQ24" t="inlineStr">
@@ -4976,27 +4976,27 @@
       </c>
       <c r="AR24" t="inlineStr">
         <is>
-          <t>1 5/16-12 (male JIC 37 deg)</t>
+          <t>1 1/16-12 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS24" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -12 (O 1.625)</t>
+          <t>SAE code 62 flange head -20 (O 2.125)</t>
         </is>
       </c>
       <c r="AT24" t="inlineStr">
         <is>
-          <t>2.930</t>
+          <t>2.830</t>
         </is>
       </c>
       <c r="AU24" t="inlineStr">
         <is>
-          <t>2.280</t>
+          <t>2.760</t>
         </is>
       </c>
       <c r="AV24" t="inlineStr">
         <is>
-          <t>1.253</t>
+          <t>1.258</t>
         </is>
       </c>
       <c r="AW24" t="inlineStr">
@@ -5011,24 +5011,24 @@
       </c>
       <c r="AY24" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-16-12 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -12: head OD / thickness / face O-ring groove measured on BRENNAN_1803-12-12.stp (= Brennan catalog 3300-62-12-12 A 1.625 / D 0.345 / H 1.250); single manufacturer - SAE J518 / ISO 6162-2 not in the repo; edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-12-20 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -20: head OD 2.125 / thickness 0.405 / groove OD 1.750 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.440 / depth 0.11 = the code 61 -20 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-16-12: L1 2.93 L2 2.28 AF 1.375 JT 0.453 GT 0.911 AFL 1.625 EFL 0.345 BFL 1.25 DFL 1.26 FFL 0.709 DRILLFL 0.551 TOD 0.8 EXT 1.566 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-12-20: L1 2.83 L2 2.76 AF 1.125 JT 0.394 GT 0.864 AFL 2.125 EFL 0.405 BFL 1.75 DFL 1.732 FFL 0.984 DRILLFL 0.551 TOD 0.8 EXT 1.572 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA24" t="inlineStr">
         <is>
-          <t>1804-16-12-Tube</t>
+          <t>1804-12-20-Tube</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1804-16-16-Tube</t>
+          <t>1804-16-12-Tube</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -5092,70 +5092,70 @@
         <v>0.9109969999999999</v>
       </c>
       <c r="V25" t="n">
-        <v>1.7692</v>
+        <v>1.6772</v>
       </c>
       <c r="W25" t="n">
-        <v>1.6208</v>
+        <v>1.2528</v>
       </c>
       <c r="X25" t="n">
-        <v>3.39</v>
+        <v>2.93</v>
       </c>
       <c r="Y25" t="n">
-        <v>2.11</v>
+        <v>1.621</v>
       </c>
       <c r="Z25" t="n">
-        <v>1.03</v>
+        <v>0.8</v>
       </c>
       <c r="AA25" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AB25" t="n">
         <v>0.625</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>0.78</v>
       </c>
       <c r="AC25" t="n">
         <v>0.11</v>
       </c>
       <c r="AD25" t="n">
-        <v>0.9375</v>
+        <v>0.8125</v>
       </c>
       <c r="AE25" t="n">
-        <v>0.375</v>
+        <v>0.345</v>
       </c>
       <c r="AF25" t="n">
-        <v>0.745</v>
+        <v>0.63</v>
       </c>
       <c r="AG25" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.709</v>
       </c>
       <c r="AH25" t="n">
-        <v>0.76</v>
+        <v>0.659</v>
       </c>
       <c r="AI25" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ25" t="n">
-        <v>1.7692</v>
+        <v>1.6772</v>
       </c>
       <c r="AK25" t="n">
-        <v>1.6208</v>
+        <v>1.2528</v>
       </c>
       <c r="AL25" t="n">
-        <v>3.39</v>
+        <v>2.93</v>
       </c>
       <c r="AM25" t="n">
-        <v>2.92</v>
+        <v>2.33</v>
       </c>
       <c r="AN25" t="n">
-        <v>0.74</v>
+        <v>0.551</v>
       </c>
       <c r="AO25" t="inlineStr">
         <is>
-          <t>1804-16-16-Tube</t>
+          <t>1804-16-12-Tube</t>
         </is>
       </c>
       <c r="AP25" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -16 x code 62 flange -16</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -16 x code 62 flange -12</t>
         </is>
       </c>
       <c r="AQ25" t="inlineStr">
@@ -5170,27 +5170,27 @@
       </c>
       <c r="AS25" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -16 (O 1.875)</t>
+          <t>SAE code 62 flange head -12 (O 1.625)</t>
         </is>
       </c>
       <c r="AT25" t="inlineStr">
         <is>
-          <t>3.390</t>
+          <t>2.930</t>
         </is>
       </c>
       <c r="AU25" t="inlineStr">
         <is>
-          <t>2.870</t>
+          <t>2.280</t>
         </is>
       </c>
       <c r="AV25" t="inlineStr">
         <is>
-          <t>1.621</t>
+          <t>1.253</t>
         </is>
       </c>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>1.030</t>
+          <t>0.800</t>
         </is>
       </c>
       <c r="AX25" t="inlineStr">
@@ -5200,24 +5200,24 @@
       </c>
       <c r="AY25" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-16-16 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -16: head OD 1.875 / thickness 0.375 / groove OD 1.560 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.250 / depth 0.11 = the code 61 -16 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-16-12 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -12: head OD / thickness / face O-ring groove measured on BRENNAN_1803-12-12.stp (= Brennan catalog 3300-62-12-12 A 1.625 / D 0.345 / H 1.250); single manufacturer - SAE J518 / ISO 6162-2 not in the repo; edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-16-16: L1 3.39 L2 2.87 AF 1.375 JT 0.453 GT 0.911 AFL 1.875 EFL 0.375 BFL 1.56 DFL 1.49 FFL 0.81 DRILLFL 0.74 TOD 1.03 EXT 2.026 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-16-12: L1 2.93 L2 2.28 AF 1.375 JT 0.453 GT 0.911 AFL 1.625 EFL 0.345 BFL 1.25 DFL 1.26 FFL 0.709 DRILLFL 0.551 TOD 0.8 EXT 1.566 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA25" t="inlineStr">
         <is>
-          <t>1804-16-16-Tube</t>
+          <t>1804-16-12-Tube</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1804-16-20-Tube</t>
+          <t>1804-16-16-Tube</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -5290,34 +5290,34 @@
         <v>3.39</v>
       </c>
       <c r="Y26" t="n">
-        <v>2.096</v>
+        <v>2.11</v>
       </c>
       <c r="Z26" t="n">
-        <v>1.043</v>
+        <v>1.03</v>
       </c>
       <c r="AA26" t="n">
-        <v>0.72</v>
+        <v>0.625</v>
       </c>
       <c r="AB26" t="n">
-        <v>0.875</v>
+        <v>0.78</v>
       </c>
       <c r="AC26" t="n">
         <v>0.11</v>
       </c>
       <c r="AD26" t="n">
-        <v>1.0625</v>
+        <v>0.9375</v>
       </c>
       <c r="AE26" t="n">
-        <v>0.405</v>
+        <v>0.375</v>
       </c>
       <c r="AF26" t="n">
-        <v>0.866</v>
+        <v>0.745</v>
       </c>
       <c r="AG26" t="n">
-        <v>0.984</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AH26" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.76</v>
       </c>
       <c r="AI26" t="n">
         <v>0.05</v>
@@ -5332,19 +5332,19 @@
         <v>3.39</v>
       </c>
       <c r="AM26" t="n">
-        <v>3.08</v>
+        <v>2.92</v>
       </c>
       <c r="AN26" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="AO26" t="inlineStr">
         <is>
-          <t>1804-16-20-Tube</t>
+          <t>1804-16-16-Tube</t>
         </is>
       </c>
       <c r="AP26" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -16 x code 62 flange -20</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -16 x code 62 flange -16</t>
         </is>
       </c>
       <c r="AQ26" t="inlineStr">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="AS26" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -20 (O 2.125)</t>
+          <t>SAE code 62 flange head -16 (O 1.875)</t>
         </is>
       </c>
       <c r="AT26" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="AU26" t="inlineStr">
         <is>
-          <t>3.030</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="AV26" t="inlineStr">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>1.043</t>
+          <t>1.030</t>
         </is>
       </c>
       <c r="AX26" t="inlineStr">
@@ -5389,49 +5389,49 @@
       </c>
       <c r="AY26" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-16-20 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -20: head OD 2.125 / thickness 0.405 / groove OD 1.750 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.440 / depth 0.11 = the code 61 -20 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-16-16 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -16: head OD 1.875 / thickness 0.375 / groove OD 1.560 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.250 / depth 0.11 = the code 61 -16 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-16-20: L1 3.39 L2 3.03 AF 1.375 JT 0.453 GT 0.911 AFL 2.125 EFL 0.405 BFL 1.75 DFL 1.732 FFL 0.984 DRILLFL 0.75 TOD 1.043 EXT 2.026 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-16-16: L1 3.39 L2 2.87 AF 1.375 JT 0.453 GT 0.911 AFL 1.875 EFL 0.375 BFL 1.56 DFL 1.49 FFL 0.81 DRILLFL 0.74 TOD 1.03 EXT 2.026 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA26" t="inlineStr">
         <is>
-          <t>1804-16-20-Tube</t>
+          <t>1804-16-16-Tube</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1804-20-16-Tube</t>
+          <t>1804-16-20-Tube</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1.488952</v>
+        <v>1.363997</v>
       </c>
       <c r="C27" t="n">
-        <v>0.974279</v>
+        <v>0.793857</v>
       </c>
       <c r="D27" t="n">
-        <v>0.8125</v>
+        <v>0.65625</v>
       </c>
       <c r="E27" t="n">
         <v>0.125</v>
       </c>
       <c r="F27" t="n">
-        <v>0.4316</v>
+        <v>0.4365</v>
       </c>
       <c r="G27" t="n">
-        <v>0.753</v>
+        <v>0.5965</v>
       </c>
       <c r="H27" t="n">
-        <v>0.1288</v>
+        <v>0.1292</v>
       </c>
       <c r="I27" t="n">
-        <v>0.2382</v>
+        <v>0.1858</v>
       </c>
       <c r="J27" t="n">
         <v>60</v>
@@ -5440,13 +5440,13 @@
         <v>37</v>
       </c>
       <c r="L27" t="n">
-        <v>1.625</v>
+        <v>1.3125</v>
       </c>
       <c r="M27" t="n">
         <v>0.08333</v>
       </c>
       <c r="N27" t="n">
-        <v>0.7986</v>
+        <v>0.7514999999999999</v>
       </c>
       <c r="O27" t="n">
         <v>0.04511</v>
@@ -5458,82 +5458,82 @@
         <v>0.08333</v>
       </c>
       <c r="R27" t="n">
-        <v>1.6875</v>
+        <v>1.375</v>
       </c>
       <c r="S27" t="n">
-        <v>0.957952</v>
+        <v>0.9109969999999999</v>
       </c>
       <c r="T27" t="n">
-        <v>0.531</v>
+        <v>0.453</v>
       </c>
       <c r="U27" t="n">
-        <v>0.957952</v>
+        <v>0.9109969999999999</v>
       </c>
       <c r="V27" t="n">
-        <v>1.9056</v>
+        <v>1.7692</v>
       </c>
       <c r="W27" t="n">
-        <v>1.6344</v>
+        <v>1.6208</v>
       </c>
       <c r="X27" t="n">
-        <v>3.54</v>
+        <v>3.39</v>
       </c>
       <c r="Y27" t="n">
-        <v>2.093</v>
+        <v>2.096</v>
       </c>
       <c r="Z27" t="n">
         <v>1.043</v>
       </c>
       <c r="AA27" t="n">
-        <v>0.625</v>
+        <v>0.72</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.78</v>
+        <v>0.875</v>
       </c>
       <c r="AC27" t="n">
         <v>0.11</v>
       </c>
       <c r="AD27" t="n">
-        <v>0.9375</v>
+        <v>1.0625</v>
       </c>
       <c r="AE27" t="n">
-        <v>0.375</v>
+        <v>0.405</v>
       </c>
       <c r="AF27" t="n">
-        <v>0.748</v>
+        <v>0.866</v>
       </c>
       <c r="AG27" t="n">
-        <v>0.827</v>
+        <v>0.984</v>
       </c>
       <c r="AH27" t="n">
-        <v>0.777</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="AI27" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ27" t="n">
-        <v>1.9056</v>
+        <v>1.7692</v>
       </c>
       <c r="AK27" t="n">
-        <v>1.6344</v>
+        <v>1.6208</v>
       </c>
       <c r="AL27" t="n">
-        <v>3.54</v>
+        <v>3.39</v>
       </c>
       <c r="AM27" t="n">
-        <v>2.92</v>
+        <v>3.08</v>
       </c>
       <c r="AN27" t="n">
         <v>0.75</v>
       </c>
       <c r="AO27" t="inlineStr">
         <is>
-          <t>1804-20-16-Tube</t>
+          <t>1804-16-20-Tube</t>
         </is>
       </c>
       <c r="AP27" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 62 flange -16</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -16 x code 62 flange -20</t>
         </is>
       </c>
       <c r="AQ27" t="inlineStr">
@@ -5543,27 +5543,27 @@
       </c>
       <c r="AR27" t="inlineStr">
         <is>
-          <t>1 5/8-12 (male JIC 37 deg)</t>
+          <t>1 5/16-12 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS27" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -16 (O 1.875)</t>
+          <t>SAE code 62 flange head -20 (O 2.125)</t>
         </is>
       </c>
       <c r="AT27" t="inlineStr">
         <is>
-          <t>3.540</t>
+          <t>3.390</t>
         </is>
       </c>
       <c r="AU27" t="inlineStr">
         <is>
-          <t>2.870</t>
+          <t>3.030</t>
         </is>
       </c>
       <c r="AV27" t="inlineStr">
         <is>
-          <t>1.634</t>
+          <t>1.621</t>
         </is>
       </c>
       <c r="AW27" t="inlineStr">
@@ -5578,49 +5578,49 @@
       </c>
       <c r="AY27" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-20-16 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -16: head OD 1.875 / thickness 0.375 / groove OD 1.560 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.250 / depth 0.11 = the code 61 -16 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-16-20 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -20: head OD 2.125 / thickness 0.405 / groove OD 1.750 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.440 / depth 0.11 = the code 61 -20 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-20-16: L1 3.54 L2 2.87 AF 1.6875 JT 0.531 GT 0.958 AFL 1.875 EFL 0.375 BFL 1.56 DFL 1.496 FFL 0.827 DRILLFL 0.75 TOD 1.043 EXT 2.043 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-16-20: L1 3.39 L2 3.03 AF 1.375 JT 0.453 GT 0.911 AFL 2.125 EFL 0.405 BFL 1.75 DFL 1.732 FFL 0.984 DRILLFL 0.75 TOD 1.043 EXT 2.026 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA27" t="inlineStr">
         <is>
-          <t>1804-20-16-Tube</t>
+          <t>1804-16-20-Tube</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1804-20-20-Tube</t>
+          <t>1804-16-24-Tube</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1.488952</v>
+        <v>1.363997</v>
       </c>
       <c r="C28" t="n">
-        <v>0.974279</v>
+        <v>0.793857</v>
       </c>
       <c r="D28" t="n">
-        <v>0.8125</v>
+        <v>0.65625</v>
       </c>
       <c r="E28" t="n">
         <v>0.125</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4316</v>
+        <v>0.4365</v>
       </c>
       <c r="G28" t="n">
-        <v>0.753</v>
+        <v>0.5965</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1288</v>
+        <v>0.1292</v>
       </c>
       <c r="I28" t="n">
-        <v>0.2382</v>
+        <v>0.1858</v>
       </c>
       <c r="J28" t="n">
         <v>60</v>
@@ -5629,13 +5629,13 @@
         <v>37</v>
       </c>
       <c r="L28" t="n">
-        <v>1.625</v>
+        <v>1.3125</v>
       </c>
       <c r="M28" t="n">
         <v>0.08333</v>
       </c>
       <c r="N28" t="n">
-        <v>0.7986</v>
+        <v>0.7514999999999999</v>
       </c>
       <c r="O28" t="n">
         <v>0.04511</v>
@@ -5647,82 +5647,82 @@
         <v>0.08333</v>
       </c>
       <c r="R28" t="n">
-        <v>1.6875</v>
+        <v>1.375</v>
       </c>
       <c r="S28" t="n">
-        <v>0.957952</v>
+        <v>0.9109969999999999</v>
       </c>
       <c r="T28" t="n">
-        <v>0.531</v>
+        <v>0.453</v>
       </c>
       <c r="U28" t="n">
-        <v>0.957952</v>
+        <v>0.9109969999999999</v>
       </c>
       <c r="V28" t="n">
-        <v>1.9992</v>
+        <v>1.7692</v>
       </c>
       <c r="W28" t="n">
-        <v>1.9808</v>
+        <v>1.6208</v>
       </c>
       <c r="X28" t="n">
-        <v>3.98</v>
+        <v>3.39</v>
       </c>
       <c r="Y28" t="n">
-        <v>2.526</v>
+        <v>2.099</v>
       </c>
       <c r="Z28" t="n">
-        <v>1.339</v>
+        <v>0.8</v>
       </c>
       <c r="AA28" t="n">
-        <v>0.72</v>
+        <v>0.9025</v>
       </c>
       <c r="AB28" t="n">
-        <v>0.875</v>
+        <v>1.0575</v>
       </c>
       <c r="AC28" t="n">
         <v>0.11</v>
       </c>
       <c r="AD28" t="n">
-        <v>1.0625</v>
+        <v>1.25</v>
       </c>
       <c r="AE28" t="n">
-        <v>0.405</v>
+        <v>0.495</v>
       </c>
       <c r="AF28" t="n">
-        <v>0.866</v>
+        <v>1.004</v>
       </c>
       <c r="AG28" t="n">
-        <v>0.984</v>
+        <v>1.181</v>
       </c>
       <c r="AH28" t="n">
-        <v>0.9340000000000001</v>
+        <v>1.131</v>
       </c>
       <c r="AI28" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ28" t="n">
-        <v>1.9992</v>
+        <v>1.7692</v>
       </c>
       <c r="AK28" t="n">
-        <v>1.9808</v>
+        <v>1.6208</v>
       </c>
       <c r="AL28" t="n">
-        <v>3.98</v>
+        <v>3.39</v>
       </c>
       <c r="AM28" t="n">
-        <v>3.51</v>
+        <v>3.28</v>
       </c>
       <c r="AN28" t="n">
-        <v>1.004</v>
+        <v>0.74</v>
       </c>
       <c r="AO28" t="inlineStr">
         <is>
-          <t>1804-20-20-Tube</t>
+          <t>1804-16-24-Tube</t>
         </is>
       </c>
       <c r="AP28" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 62 flange -20</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -16 x code 62 flange -24</t>
         </is>
       </c>
       <c r="AQ28" t="inlineStr">
@@ -5732,32 +5732,32 @@
       </c>
       <c r="AR28" t="inlineStr">
         <is>
-          <t>1 5/8-12 (male JIC 37 deg)</t>
+          <t>1 5/16-12 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS28" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -20 (O 2.125)</t>
+          <t>SAE code 62 flange head -24 (O 2.5)</t>
         </is>
       </c>
       <c r="AT28" t="inlineStr">
         <is>
-          <t>3.980</t>
+          <t>3.390</t>
         </is>
       </c>
       <c r="AU28" t="inlineStr">
         <is>
-          <t>3.460</t>
+          <t>3.230</t>
         </is>
       </c>
       <c r="AV28" t="inlineStr">
         <is>
-          <t>1.981</t>
+          <t>1.621</t>
         </is>
       </c>
       <c r="AW28" t="inlineStr">
         <is>
-          <t>1.339</t>
+          <t>0.800</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr">
@@ -5767,24 +5767,24 @@
       </c>
       <c r="AY28" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-20-20 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -20: head OD 2.125 / thickness 0.405 / groove OD 1.750 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.440 / depth 0.11 = the code 61 -20 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-16-24 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -24: head OD 2.5 / thickness 0.495 / groove OD 2.115 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.805 / depth 0.11 = the code 61 -24 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-20-20: L1 3.98 L2 3.46 AF 1.6875 JT 0.531 GT 0.958 AFL 2.125 EFL 0.405 BFL 1.75 DFL 1.732 FFL 0.984 DRILLFL 1.004 TOD 1.339 EXT 2.476 (codes: README s2). </t>
+          <t>Brennan record 1804-16-24: L1 3.39 L2 3.23 AF 1.375 JT 0.453 GT 0.911 AFL 2.5 EFL 0.495 BFL 2.115 DFL 2.008 FFL 1.181 DRILLFL 0.74 TOD 0.8 EXT 2.026 (codes: README s2).  BRENNAN_1804-16-24.stp confirms the record: tube 0.800 / bore 0.740 (bend torus tube dia 0.800 / 0.740, R 1.6208 = 0.8 x EXT) - a 0.030 wall, built as Brennan models it (the other -16 JIC rows have a 1.043 tube).</t>
         </is>
       </c>
       <c r="BA28" t="inlineStr">
         <is>
-          <t>1804-20-20-Tube</t>
+          <t>1804-16-24-Tube</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1804-20-24-Tube</t>
+          <t>1804-20-16-Tube</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -5848,70 +5848,70 @@
         <v>0.957952</v>
       </c>
       <c r="V29" t="n">
-        <v>1.9968</v>
+        <v>1.9056</v>
       </c>
       <c r="W29" t="n">
-        <v>1.9832</v>
+        <v>1.6344</v>
       </c>
       <c r="X29" t="n">
-        <v>3.98</v>
+        <v>3.54</v>
       </c>
       <c r="Y29" t="n">
-        <v>2.529</v>
+        <v>2.093</v>
       </c>
       <c r="Z29" t="n">
-        <v>1.339</v>
+        <v>1.043</v>
       </c>
       <c r="AA29" t="n">
-        <v>0.9025</v>
+        <v>0.625</v>
       </c>
       <c r="AB29" t="n">
-        <v>1.0575</v>
+        <v>0.78</v>
       </c>
       <c r="AC29" t="n">
         <v>0.11</v>
       </c>
       <c r="AD29" t="n">
-        <v>1.25</v>
+        <v>0.9375</v>
       </c>
       <c r="AE29" t="n">
-        <v>0.495</v>
+        <v>0.375</v>
       </c>
       <c r="AF29" t="n">
-        <v>1.004</v>
+        <v>0.748</v>
       </c>
       <c r="AG29" t="n">
-        <v>1.181</v>
+        <v>0.827</v>
       </c>
       <c r="AH29" t="n">
-        <v>1.131</v>
+        <v>0.777</v>
       </c>
       <c r="AI29" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ29" t="n">
-        <v>1.9968</v>
+        <v>1.9056</v>
       </c>
       <c r="AK29" t="n">
-        <v>1.9832</v>
+        <v>1.6344</v>
       </c>
       <c r="AL29" t="n">
-        <v>3.98</v>
+        <v>3.54</v>
       </c>
       <c r="AM29" t="n">
-        <v>3.71</v>
+        <v>2.92</v>
       </c>
       <c r="AN29" t="n">
-        <v>0.975</v>
+        <v>0.75</v>
       </c>
       <c r="AO29" t="inlineStr">
         <is>
-          <t>1804-20-24-Tube</t>
+          <t>1804-20-16-Tube</t>
         </is>
       </c>
       <c r="AP29" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 62 flange -24</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 62 flange -16</t>
         </is>
       </c>
       <c r="AQ29" t="inlineStr">
@@ -5926,27 +5926,27 @@
       </c>
       <c r="AS29" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -24 (O 2.5)</t>
+          <t>SAE code 62 flange head -16 (O 1.875)</t>
         </is>
       </c>
       <c r="AT29" t="inlineStr">
         <is>
-          <t>3.980</t>
+          <t>3.540</t>
         </is>
       </c>
       <c r="AU29" t="inlineStr">
         <is>
-          <t>3.660</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="AV29" t="inlineStr">
         <is>
-          <t>1.983</t>
+          <t>1.634</t>
         </is>
       </c>
       <c r="AW29" t="inlineStr">
         <is>
-          <t>1.339</t>
+          <t>1.043</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr">
@@ -5956,49 +5956,49 @@
       </c>
       <c r="AY29" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-20-24 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -24: head OD 2.5 / thickness 0.495 / groove OD 2.115 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.805 / depth 0.11 = the code 61 -24 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-20-16 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -16: head OD 1.875 / thickness 0.375 / groove OD 1.560 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.250 / depth 0.11 = the code 61 -16 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-20-24: L1 3.98 L2 3.66 AF 1.6875 JT 0.531 GT 0.958 AFL 2.5 EFL 0.495 BFL 2.115 DFL 2.008 FFL 1.181 DRILLFL 0.975 TOD 1.339 EXT 2.479 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-20-16: L1 3.54 L2 2.87 AF 1.6875 JT 0.531 GT 0.958 AFL 1.875 EFL 0.375 BFL 1.56 DFL 1.496 FFL 0.827 DRILLFL 0.75 TOD 1.043 EXT 2.043 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA29" t="inlineStr">
         <is>
-          <t>1804-20-24-Tube</t>
+          <t>1804-20-16-Tube</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1804-24-16-Tube</t>
+          <t>1804-20-20-Tube</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.713041</v>
+        <v>1.488952</v>
       </c>
       <c r="C30" t="n">
-        <v>1.154701</v>
+        <v>0.974279</v>
       </c>
       <c r="D30" t="n">
-        <v>0.9375</v>
+        <v>0.8125</v>
       </c>
       <c r="E30" t="n">
         <v>0.125</v>
       </c>
       <c r="F30" t="n">
-        <v>0.5454</v>
+        <v>0.4316</v>
       </c>
       <c r="G30" t="n">
-        <v>0.8774999999999999</v>
+        <v>0.753</v>
       </c>
       <c r="H30" t="n">
-        <v>0.1298</v>
+        <v>0.1288</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2482</v>
+        <v>0.2382</v>
       </c>
       <c r="J30" t="n">
         <v>60</v>
@@ -6007,13 +6007,13 @@
         <v>37</v>
       </c>
       <c r="L30" t="n">
-        <v>1.875</v>
+        <v>1.625</v>
       </c>
       <c r="M30" t="n">
         <v>0.08333</v>
       </c>
       <c r="N30" t="n">
-        <v>0.9234</v>
+        <v>0.7986</v>
       </c>
       <c r="O30" t="n">
         <v>0.04511</v>
@@ -6025,82 +6025,82 @@
         <v>0.08333</v>
       </c>
       <c r="R30" t="n">
-        <v>2</v>
+        <v>1.6875</v>
       </c>
       <c r="S30" t="n">
-        <v>1.083041</v>
+        <v>0.957952</v>
       </c>
       <c r="T30" t="n">
-        <v>0.63</v>
+        <v>0.531</v>
       </c>
       <c r="U30" t="n">
-        <v>1.083041</v>
+        <v>0.957952</v>
       </c>
       <c r="V30" t="n">
-        <v>2.3056</v>
+        <v>1.9992</v>
       </c>
       <c r="W30" t="n">
-        <v>1.6344</v>
+        <v>1.9808</v>
       </c>
       <c r="X30" t="n">
-        <v>3.94</v>
+        <v>3.98</v>
       </c>
       <c r="Y30" t="n">
-        <v>2.093</v>
+        <v>2.526</v>
       </c>
       <c r="Z30" t="n">
         <v>1.339</v>
       </c>
       <c r="AA30" t="n">
-        <v>0.625</v>
+        <v>0.72</v>
       </c>
       <c r="AB30" t="n">
-        <v>0.78</v>
+        <v>0.875</v>
       </c>
       <c r="AC30" t="n">
         <v>0.11</v>
       </c>
       <c r="AD30" t="n">
-        <v>0.9375</v>
+        <v>1.0625</v>
       </c>
       <c r="AE30" t="n">
-        <v>0.375</v>
+        <v>0.405</v>
       </c>
       <c r="AF30" t="n">
-        <v>0.748</v>
+        <v>0.866</v>
       </c>
       <c r="AG30" t="n">
-        <v>0.827</v>
+        <v>0.984</v>
       </c>
       <c r="AH30" t="n">
-        <v>0.777</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="AI30" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ30" t="n">
-        <v>2.3056</v>
+        <v>1.9992</v>
       </c>
       <c r="AK30" t="n">
-        <v>1.6344</v>
+        <v>1.9808</v>
       </c>
       <c r="AL30" t="n">
-        <v>3.94</v>
+        <v>3.98</v>
       </c>
       <c r="AM30" t="n">
-        <v>2.92</v>
+        <v>3.51</v>
       </c>
       <c r="AN30" t="n">
-        <v>0.74</v>
+        <v>1.004</v>
       </c>
       <c r="AO30" t="inlineStr">
         <is>
-          <t>1804-24-16-Tube</t>
+          <t>1804-20-20-Tube</t>
         </is>
       </c>
       <c r="AP30" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 62 flange -16</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 62 flange -20</t>
         </is>
       </c>
       <c r="AQ30" t="inlineStr">
@@ -6110,27 +6110,27 @@
       </c>
       <c r="AR30" t="inlineStr">
         <is>
-          <t>1 7/8-12 (male JIC 37 deg)</t>
+          <t>1 5/8-12 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS30" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -16 (O 1.875)</t>
+          <t>SAE code 62 flange head -20 (O 2.125)</t>
         </is>
       </c>
       <c r="AT30" t="inlineStr">
         <is>
-          <t>3.940</t>
+          <t>3.980</t>
         </is>
       </c>
       <c r="AU30" t="inlineStr">
         <is>
-          <t>2.870</t>
+          <t>3.460</t>
         </is>
       </c>
       <c r="AV30" t="inlineStr">
         <is>
-          <t>1.634</t>
+          <t>1.981</t>
         </is>
       </c>
       <c r="AW30" t="inlineStr">
@@ -6145,49 +6145,49 @@
       </c>
       <c r="AY30" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-24-16 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -16: head OD 1.875 / thickness 0.375 / groove OD 1.560 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.250 / depth 0.11 = the code 61 -16 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-20-20 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -20: head OD 2.125 / thickness 0.405 / groove OD 1.750 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.440 / depth 0.11 = the code 61 -20 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-24-16: L1 3.94 L2 2.87 AF 2.0 JT 0.63 GT 1.083 AFL 1.875 EFL 0.375 BFL 1.56 DFL 1.496 FFL 0.827 DRILLFL 0.74 TOD 1.339 EXT 2.043 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-20-20: L1 3.98 L2 3.46 AF 1.6875 JT 0.531 GT 0.958 AFL 2.125 EFL 0.405 BFL 1.75 DFL 1.732 FFL 0.984 DRILLFL 1.004 TOD 1.339 EXT 2.476 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA30" t="inlineStr">
         <is>
-          <t>1804-24-16-Tube</t>
+          <t>1804-20-20-Tube</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1804-24-20-Tube</t>
+          <t>1804-20-24-Tube</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1.713041</v>
+        <v>1.488952</v>
       </c>
       <c r="C31" t="n">
-        <v>1.154701</v>
+        <v>0.974279</v>
       </c>
       <c r="D31" t="n">
-        <v>0.9375</v>
+        <v>0.8125</v>
       </c>
       <c r="E31" t="n">
         <v>0.125</v>
       </c>
       <c r="F31" t="n">
-        <v>0.5454</v>
+        <v>0.4316</v>
       </c>
       <c r="G31" t="n">
-        <v>0.8774999999999999</v>
+        <v>0.753</v>
       </c>
       <c r="H31" t="n">
-        <v>0.1298</v>
+        <v>0.1288</v>
       </c>
       <c r="I31" t="n">
-        <v>0.2482</v>
+        <v>0.2382</v>
       </c>
       <c r="J31" t="n">
         <v>60</v>
@@ -6196,13 +6196,13 @@
         <v>37</v>
       </c>
       <c r="L31" t="n">
-        <v>1.875</v>
+        <v>1.625</v>
       </c>
       <c r="M31" t="n">
         <v>0.08333</v>
       </c>
       <c r="N31" t="n">
-        <v>0.9234</v>
+        <v>0.7986</v>
       </c>
       <c r="O31" t="n">
         <v>0.04511</v>
@@ -6214,82 +6214,82 @@
         <v>0.08333</v>
       </c>
       <c r="R31" t="n">
-        <v>2</v>
+        <v>1.6875</v>
       </c>
       <c r="S31" t="n">
-        <v>1.083041</v>
+        <v>0.957952</v>
       </c>
       <c r="T31" t="n">
-        <v>0.63</v>
+        <v>0.531</v>
       </c>
       <c r="U31" t="n">
-        <v>1.083041</v>
+        <v>0.957952</v>
       </c>
       <c r="V31" t="n">
-        <v>2.3492</v>
+        <v>1.9968</v>
       </c>
       <c r="W31" t="n">
-        <v>1.9808</v>
+        <v>1.9832</v>
       </c>
       <c r="X31" t="n">
-        <v>4.33</v>
+        <v>3.98</v>
       </c>
       <c r="Y31" t="n">
-        <v>2.526</v>
+        <v>2.529</v>
       </c>
       <c r="Z31" t="n">
         <v>1.339</v>
       </c>
       <c r="AA31" t="n">
-        <v>0.72</v>
+        <v>0.9025</v>
       </c>
       <c r="AB31" t="n">
-        <v>0.875</v>
+        <v>1.0575</v>
       </c>
       <c r="AC31" t="n">
         <v>0.11</v>
       </c>
       <c r="AD31" t="n">
-        <v>1.0625</v>
+        <v>1.25</v>
       </c>
       <c r="AE31" t="n">
-        <v>0.405</v>
+        <v>0.495</v>
       </c>
       <c r="AF31" t="n">
-        <v>0.866</v>
+        <v>1.004</v>
       </c>
       <c r="AG31" t="n">
-        <v>0.984</v>
+        <v>1.181</v>
       </c>
       <c r="AH31" t="n">
-        <v>0.9340000000000001</v>
+        <v>1.131</v>
       </c>
       <c r="AI31" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ31" t="n">
-        <v>2.3492</v>
+        <v>1.9968</v>
       </c>
       <c r="AK31" t="n">
-        <v>1.9808</v>
+        <v>1.9832</v>
       </c>
       <c r="AL31" t="n">
-        <v>4.33</v>
+        <v>3.98</v>
       </c>
       <c r="AM31" t="n">
-        <v>3.51</v>
+        <v>3.71</v>
       </c>
       <c r="AN31" t="n">
-        <v>1.004</v>
+        <v>0.975</v>
       </c>
       <c r="AO31" t="inlineStr">
         <is>
-          <t>1804-24-20-Tube</t>
+          <t>1804-20-24-Tube</t>
         </is>
       </c>
       <c r="AP31" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 62 flange -20</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -20 x code 62 flange -24</t>
         </is>
       </c>
       <c r="AQ31" t="inlineStr">
@@ -6299,27 +6299,27 @@
       </c>
       <c r="AR31" t="inlineStr">
         <is>
-          <t>1 7/8-12 (male JIC 37 deg)</t>
+          <t>1 5/8-12 (male JIC 37 deg)</t>
         </is>
       </c>
       <c r="AS31" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -20 (O 2.125)</t>
+          <t>SAE code 62 flange head -24 (O 2.5)</t>
         </is>
       </c>
       <c r="AT31" t="inlineStr">
         <is>
-          <t>4.330</t>
+          <t>3.980</t>
         </is>
       </c>
       <c r="AU31" t="inlineStr">
         <is>
-          <t>3.460</t>
+          <t>3.660</t>
         </is>
       </c>
       <c r="AV31" t="inlineStr">
         <is>
-          <t>1.981</t>
+          <t>1.983</t>
         </is>
       </c>
       <c r="AW31" t="inlineStr">
@@ -6334,24 +6334,24 @@
       </c>
       <c r="AY31" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-24-20 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -20: head OD 2.125 / thickness 0.405 / groove OD 1.750 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.440 / depth 0.11 = the code 61 -20 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-20-24 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -24: head OD 2.5 / thickness 0.495 / groove OD 2.115 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.805 / depth 0.11 = the code 61 -24 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-24-20: L1 4.33 L2 3.46 AF 2.0 JT 0.63 GT 1.083 AFL 2.125 EFL 0.405 BFL 1.75 DFL 1.732 FFL 0.984 DRILLFL 1.004 TOD 1.339 EXT 2.476 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-20-24: L1 3.98 L2 3.66 AF 1.6875 JT 0.531 GT 0.958 AFL 2.5 EFL 0.495 BFL 2.115 DFL 2.008 FFL 1.181 DRILLFL 0.975 TOD 1.339 EXT 2.479 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA31" t="inlineStr">
         <is>
-          <t>1804-24-20-Tube</t>
+          <t>1804-20-24-Tube</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1804-24-24-Tube</t>
+          <t>1804-24-16-Tube</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -6415,70 +6415,70 @@
         <v>1.083041</v>
       </c>
       <c r="V32" t="n">
-        <v>2.2988</v>
+        <v>2.3056</v>
       </c>
       <c r="W32" t="n">
-        <v>2.2712</v>
+        <v>1.6344</v>
       </c>
       <c r="X32" t="n">
-        <v>4.57</v>
+        <v>3.94</v>
       </c>
       <c r="Y32" t="n">
-        <v>2.889</v>
+        <v>2.093</v>
       </c>
       <c r="Z32" t="n">
-        <v>1.575</v>
+        <v>1.339</v>
       </c>
       <c r="AA32" t="n">
-        <v>0.9025</v>
+        <v>0.625</v>
       </c>
       <c r="AB32" t="n">
-        <v>1.0575</v>
+        <v>0.78</v>
       </c>
       <c r="AC32" t="n">
         <v>0.11</v>
       </c>
       <c r="AD32" t="n">
-        <v>1.25</v>
+        <v>0.9375</v>
       </c>
       <c r="AE32" t="n">
-        <v>0.495</v>
+        <v>0.375</v>
       </c>
       <c r="AF32" t="n">
-        <v>1.004</v>
+        <v>0.748</v>
       </c>
       <c r="AG32" t="n">
-        <v>1.181</v>
+        <v>0.827</v>
       </c>
       <c r="AH32" t="n">
-        <v>1.131</v>
+        <v>0.777</v>
       </c>
       <c r="AI32" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ32" t="n">
-        <v>2.2988</v>
+        <v>2.3056</v>
       </c>
       <c r="AK32" t="n">
-        <v>2.2712</v>
+        <v>1.6344</v>
       </c>
       <c r="AL32" t="n">
-        <v>4.57</v>
+        <v>3.94</v>
       </c>
       <c r="AM32" t="n">
-        <v>4.07</v>
+        <v>2.92</v>
       </c>
       <c r="AN32" t="n">
-        <v>1.23</v>
+        <v>0.74</v>
       </c>
       <c r="AO32" t="inlineStr">
         <is>
-          <t>1804-24-24-Tube</t>
+          <t>1804-24-16-Tube</t>
         </is>
       </c>
       <c r="AP32" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 62 flange -24</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 62 flange -16</t>
         </is>
       </c>
       <c r="AQ32" t="inlineStr">
@@ -6493,27 +6493,27 @@
       </c>
       <c r="AS32" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -24 (O 2.5)</t>
+          <t>SAE code 62 flange head -16 (O 1.875)</t>
         </is>
       </c>
       <c r="AT32" t="inlineStr">
         <is>
-          <t>4.570</t>
+          <t>3.940</t>
         </is>
       </c>
       <c r="AU32" t="inlineStr">
         <is>
-          <t>4.020</t>
+          <t>2.870</t>
         </is>
       </c>
       <c r="AV32" t="inlineStr">
         <is>
-          <t>2.271</t>
+          <t>1.634</t>
         </is>
       </c>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>1.575</t>
+          <t>1.339</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr">
@@ -6523,24 +6523,24 @@
       </c>
       <c r="AY32" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-24-24 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -24: head OD 2.5 / thickness 0.495 / groove OD 2.115 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.805 / depth 0.11 = the code 61 -24 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-24-16 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -16: head OD 1.875 / thickness 0.375 / groove OD 1.560 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.250 / depth 0.11 = the code 61 -16 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-24-24: L1 4.57 L2 4.02 AF 2.0 JT 0.63 GT 1.083 AFL 2.5 EFL 0.495 BFL 2.115 DFL 2.008 FFL 1.181 DRILLFL 1.23 TOD 1.575 EXT 2.839 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-24-16: L1 3.94 L2 2.87 AF 2.0 JT 0.63 GT 1.083 AFL 1.875 EFL 0.375 BFL 1.56 DFL 1.496 FFL 0.827 DRILLFL 0.74 TOD 1.339 EXT 2.043 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA32" t="inlineStr">
         <is>
-          <t>1804-24-24-Tube</t>
+          <t>1804-24-16-Tube</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1804-24-32-Tube</t>
+          <t>1804-24-20-Tube</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -6604,70 +6604,70 @@
         <v>1.083041</v>
       </c>
       <c r="V33" t="n">
-        <v>2.5874</v>
+        <v>2.3492</v>
       </c>
       <c r="W33" t="n">
-        <v>2.2456</v>
+        <v>1.9808</v>
       </c>
       <c r="X33" t="n">
-        <v>4.833</v>
+        <v>4.33</v>
       </c>
       <c r="Y33" t="n">
-        <v>2.857</v>
+        <v>2.526</v>
       </c>
       <c r="Z33" t="n">
-        <v>1.575</v>
+        <v>1.339</v>
       </c>
       <c r="AA33" t="n">
-        <v>1.09</v>
+        <v>0.72</v>
       </c>
       <c r="AB33" t="n">
-        <v>1.245</v>
+        <v>0.875</v>
       </c>
       <c r="AC33" t="n">
         <v>0.11</v>
       </c>
       <c r="AD33" t="n">
-        <v>1.5625</v>
+        <v>1.0625</v>
       </c>
       <c r="AE33" t="n">
-        <v>0.495</v>
+        <v>0.405</v>
       </c>
       <c r="AF33" t="n">
-        <v>1.309</v>
+        <v>0.866</v>
       </c>
       <c r="AG33" t="n">
-        <v>1.496</v>
+        <v>0.984</v>
       </c>
       <c r="AH33" t="n">
-        <v>1.446</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="AI33" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ33" t="n">
-        <v>2.5874</v>
+        <v>2.3492</v>
       </c>
       <c r="AK33" t="n">
-        <v>2.2456</v>
+        <v>1.9808</v>
       </c>
       <c r="AL33" t="n">
-        <v>4.833</v>
+        <v>4.33</v>
       </c>
       <c r="AM33" t="n">
-        <v>4.353</v>
+        <v>3.51</v>
       </c>
       <c r="AN33" t="n">
-        <v>1.23</v>
+        <v>1.004</v>
       </c>
       <c r="AO33" t="inlineStr">
         <is>
-          <t>1804-24-32-Tube</t>
+          <t>1804-24-20-Tube</t>
         </is>
       </c>
       <c r="AP33" t="inlineStr">
         <is>
-          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 62 flange -32</t>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 62 flange -20</t>
         </is>
       </c>
       <c r="AQ33" t="inlineStr">
@@ -6682,27 +6682,27 @@
       </c>
       <c r="AS33" t="inlineStr">
         <is>
-          <t>SAE code 62 flange head -32 (O 3.125)</t>
+          <t>SAE code 62 flange head -20 (O 2.125)</t>
         </is>
       </c>
       <c r="AT33" t="inlineStr">
         <is>
-          <t>4.833</t>
+          <t>4.330</t>
         </is>
       </c>
       <c r="AU33" t="inlineStr">
         <is>
-          <t>4.303</t>
+          <t>3.460</t>
         </is>
       </c>
       <c r="AV33" t="inlineStr">
         <is>
-          <t>2.246</t>
+          <t>1.981</t>
         </is>
       </c>
       <c r="AW33" t="inlineStr">
         <is>
-          <t>1.575</t>
+          <t>1.339</t>
         </is>
       </c>
       <c r="AX33" t="inlineStr">
@@ -6712,49 +6712,49 @@
       </c>
       <c r="AY33" t="inlineStr">
         <is>
-          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-24-32 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -32: head OD 3.125 / thickness 0.495 / groove OD 2.490 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 2.180 / depth 0.11 = the code 61 -32 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-24-20 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -20: head OD 2.125 / thickness 0.405 / groove OD 1.750 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.440 / depth 0.11 = the code 61 -20 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
       <c r="AZ33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brennan record 1804-24-32: L1 4.833 L2 4.303 AF 2.0 JT 0.63 GT 1.083 AFL 3.125 EFL 0.495 BFL 2.49 DFL 2.618 FFL 1.496 DRILLFL 1.23 TOD 1.575 EXT 2.807 (codes: README s2). </t>
+          <t xml:space="preserve">Brennan record 1804-24-20: L1 4.33 L2 3.46 AF 2.0 JT 0.63 GT 1.083 AFL 2.125 EFL 0.405 BFL 1.75 DFL 1.732 FFL 0.984 DRILLFL 1.004 TOD 1.339 EXT 2.476 (codes: README s2). </t>
         </is>
       </c>
       <c r="BA33" t="inlineStr">
         <is>
-          <t>1804-24-32-Tube</t>
+          <t>1804-24-20-Tube</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1804-32-32-Tube</t>
+          <t>1804-24-24-Tube</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.963041</v>
+        <v>1.713041</v>
       </c>
       <c r="C34" t="n">
-        <v>1.587713</v>
+        <v>1.154701</v>
       </c>
       <c r="D34" t="n">
-        <v>1.25</v>
+        <v>0.9375</v>
       </c>
       <c r="E34" t="n">
         <v>0.125</v>
       </c>
       <c r="F34" t="n">
-        <v>0.7124</v>
+        <v>0.5454</v>
       </c>
       <c r="G34" t="n">
-        <v>1.19</v>
+        <v>0.8774999999999999</v>
       </c>
       <c r="H34" t="n">
-        <v>0.1292</v>
+        <v>0.1298</v>
       </c>
       <c r="I34" t="n">
-        <v>0.3318</v>
+        <v>0.2482</v>
       </c>
       <c r="J34" t="n">
         <v>60</v>
@@ -6763,13 +6763,13 @@
         <v>37</v>
       </c>
       <c r="L34" t="n">
-        <v>2.5</v>
+        <v>1.875</v>
       </c>
       <c r="M34" t="n">
         <v>0.08333</v>
       </c>
       <c r="N34" t="n">
-        <v>1.1734</v>
+        <v>0.9234</v>
       </c>
       <c r="O34" t="n">
         <v>0.04511</v>
@@ -6781,135 +6781,513 @@
         <v>0.08333</v>
       </c>
       <c r="R34" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="S34" t="n">
-        <v>1.333041</v>
+        <v>1.083041</v>
       </c>
       <c r="T34" t="n">
         <v>0.63</v>
       </c>
       <c r="U34" t="n">
-        <v>1.333041</v>
+        <v>1.083041</v>
       </c>
       <c r="V34" t="n">
-        <v>2.7388</v>
+        <v>2.2988</v>
       </c>
       <c r="W34" t="n">
-        <v>3.0512</v>
+        <v>2.2712</v>
       </c>
       <c r="X34" t="n">
-        <v>5.79</v>
+        <v>4.57</v>
       </c>
       <c r="Y34" t="n">
-        <v>3.864</v>
+        <v>2.889</v>
       </c>
       <c r="Z34" t="n">
-        <v>2.087</v>
+        <v>1.575</v>
       </c>
       <c r="AA34" t="n">
-        <v>1.09</v>
+        <v>0.9025</v>
       </c>
       <c r="AB34" t="n">
-        <v>1.245</v>
+        <v>1.0575</v>
       </c>
       <c r="AC34" t="n">
         <v>0.11</v>
       </c>
       <c r="AD34" t="n">
-        <v>1.5625</v>
+        <v>1.25</v>
       </c>
       <c r="AE34" t="n">
         <v>0.495</v>
       </c>
       <c r="AF34" t="n">
-        <v>1.309</v>
+        <v>1.004</v>
       </c>
       <c r="AG34" t="n">
-        <v>1.496</v>
+        <v>1.181</v>
       </c>
       <c r="AH34" t="n">
-        <v>1.446</v>
+        <v>1.131</v>
       </c>
       <c r="AI34" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ34" t="n">
+        <v>2.2988</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>2.2712</v>
+      </c>
+      <c r="AL34" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="AO34" t="inlineStr">
+        <is>
+          <t>1804-24-24-Tube</t>
+        </is>
+      </c>
+      <c r="AP34" t="inlineStr">
+        <is>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 62 flange -24</t>
+        </is>
+      </c>
+      <c r="AQ34" t="inlineStr">
+        <is>
+          <t>1704T</t>
+        </is>
+      </c>
+      <c r="AR34" t="inlineStr">
+        <is>
+          <t>1 7/8-12 (male JIC 37 deg)</t>
+        </is>
+      </c>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>SAE code 62 flange head -24 (O 2.5)</t>
+        </is>
+      </c>
+      <c r="AT34" t="inlineStr">
+        <is>
+          <t>4.570</t>
+        </is>
+      </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>4.020</t>
+        </is>
+      </c>
+      <c r="AV34" t="inlineStr">
+        <is>
+          <t>2.271</t>
+        </is>
+      </c>
+      <c r="AW34" t="inlineStr">
+        <is>
+          <t>1.575</t>
+        </is>
+      </c>
+      <c r="AX34" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="AY34" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-24-24 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -24: head OD 2.5 / thickness 0.495 / groove OD 2.115 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 1.805 / depth 0.11 = the code 61 -24 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+        </is>
+      </c>
+      <c r="AZ34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brennan record 1804-24-24: L1 4.57 L2 4.02 AF 2.0 JT 0.63 GT 1.083 AFL 2.5 EFL 0.495 BFL 2.115 DFL 2.008 FFL 1.181 DRILLFL 1.23 TOD 1.575 EXT 2.839 (codes: README s2). </t>
+        </is>
+      </c>
+      <c r="BA34" t="inlineStr">
+        <is>
+          <t>1804-24-24-Tube</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1804-24-32-Tube</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1.713041</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1.154701</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.5454</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.8774999999999999</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.1298</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.2482</v>
+      </c>
+      <c r="J35" t="n">
+        <v>60</v>
+      </c>
+      <c r="K35" t="n">
+        <v>37</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1.875</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.9234</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0.04511</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0.02083</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="R35" t="n">
+        <v>2</v>
+      </c>
+      <c r="S35" t="n">
+        <v>1.083041</v>
+      </c>
+      <c r="T35" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="U35" t="n">
+        <v>1.083041</v>
+      </c>
+      <c r="V35" t="n">
+        <v>2.5874</v>
+      </c>
+      <c r="W35" t="n">
+        <v>2.2456</v>
+      </c>
+      <c r="X35" t="n">
+        <v>4.833</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>2.857</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>1.575</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>1.245</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>1.5625</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>1.309</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>1.496</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>1.446</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>2.5874</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>2.2456</v>
+      </c>
+      <c r="AL35" t="n">
+        <v>4.833</v>
+      </c>
+      <c r="AM35" t="n">
+        <v>4.353</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="AO35" t="inlineStr">
+        <is>
+          <t>1804-24-32-Tube</t>
+        </is>
+      </c>
+      <c r="AP35" t="inlineStr">
+        <is>
+          <t>90 deg Bent-Tube Flange Elbow, male JIC -24 x code 62 flange -32</t>
+        </is>
+      </c>
+      <c r="AQ35" t="inlineStr">
+        <is>
+          <t>1704T</t>
+        </is>
+      </c>
+      <c r="AR35" t="inlineStr">
+        <is>
+          <t>1 7/8-12 (male JIC 37 deg)</t>
+        </is>
+      </c>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>SAE code 62 flange head -32 (O 3.125)</t>
+        </is>
+      </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>4.833</t>
+        </is>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="AV35" t="inlineStr">
+        <is>
+          <t>2.246</t>
+        </is>
+      </c>
+      <c r="AW35" t="inlineStr">
+        <is>
+          <t>1.575</t>
+        </is>
+      </c>
+      <c r="AX35" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="AY35" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-24-32 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -32: head OD 3.125 / thickness 0.495 / groove OD 2.490 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 2.180 / depth 0.11 = the code 61 -32 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
+        </is>
+      </c>
+      <c r="AZ35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brennan record 1804-24-32: L1 4.833 L2 4.303 AF 2.0 JT 0.63 GT 1.083 AFL 3.125 EFL 0.495 BFL 2.49 DFL 2.618 FFL 1.496 DRILLFL 1.23 TOD 1.575 EXT 2.807 (codes: README s2). </t>
+        </is>
+      </c>
+      <c r="BA35" t="inlineStr">
+        <is>
+          <t>1804-24-32-Tube</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1804-32-32-Tube</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1.963041</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1.587713</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.7124</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.1292</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.3318</v>
+      </c>
+      <c r="J36" t="n">
+        <v>60</v>
+      </c>
+      <c r="K36" t="n">
+        <v>37</v>
+      </c>
+      <c r="L36" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="N36" t="n">
+        <v>1.1734</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.04511</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0.02083</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="R36" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="S36" t="n">
+        <v>1.333041</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="U36" t="n">
+        <v>1.333041</v>
+      </c>
+      <c r="V36" t="n">
         <v>2.7388</v>
       </c>
-      <c r="AK34" t="n">
+      <c r="W36" t="n">
         <v>3.0512</v>
       </c>
-      <c r="AL34" t="n">
+      <c r="X36" t="n">
         <v>5.79</v>
       </c>
-      <c r="AM34" t="n">
+      <c r="Y36" t="n">
+        <v>3.864</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>2.087</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>1.245</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>1.5625</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>1.309</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>1.496</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>1.446</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>2.7388</v>
+      </c>
+      <c r="AK36" t="n">
+        <v>3.0512</v>
+      </c>
+      <c r="AL36" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="AM36" t="n">
         <v>5.36</v>
       </c>
-      <c r="AN34" t="n">
+      <c r="AN36" t="n">
         <v>1.693</v>
       </c>
-      <c r="AO34" t="inlineStr">
+      <c r="AO36" t="inlineStr">
         <is>
           <t>1804-32-32-Tube</t>
         </is>
       </c>
-      <c r="AP34" t="inlineStr">
+      <c r="AP36" t="inlineStr">
         <is>
           <t>90 deg Bent-Tube Flange Elbow, male JIC -32 x code 62 flange -32</t>
         </is>
       </c>
-      <c r="AQ34" t="inlineStr">
+      <c r="AQ36" t="inlineStr">
         <is>
           <t>1704T</t>
         </is>
       </c>
-      <c r="AR34" t="inlineStr">
+      <c r="AR36" t="inlineStr">
         <is>
           <t>2 1/2-12 (male JIC 37 deg)</t>
         </is>
       </c>
-      <c r="AS34" t="inlineStr">
+      <c r="AS36" t="inlineStr">
         <is>
           <t>SAE code 62 flange head -32 (O 3.125)</t>
         </is>
       </c>
-      <c r="AT34" t="inlineStr">
+      <c r="AT36" t="inlineStr">
         <is>
           <t>5.790</t>
         </is>
       </c>
-      <c r="AU34" t="inlineStr">
+      <c r="AU36" t="inlineStr">
         <is>
           <t>5.310</t>
         </is>
       </c>
-      <c r="AV34" t="inlineStr">
+      <c r="AV36" t="inlineStr">
         <is>
           <t>3.051</t>
         </is>
       </c>
-      <c r="AW34" t="inlineStr">
+      <c r="AW36" t="inlineStr">
         <is>
           <t>2.087</t>
         </is>
       </c>
-      <c r="AX34" t="inlineStr">
+      <c r="AX36" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="AY34" t="inlineStr">
+      <c r="AY36" t="inlineStr">
         <is>
           <t>[BRENNAN-CAD 2026-10-21: M1 L1 CHEX HEXL O D TUBEOD RB HUBD HUBL] Brennan CAD record 1804-32-32 decoded on BRENNAN_1804-08-08.stp (tools/_out/groupD_20261021 README s2); 90 deg: M1 = L1, L1 = L2; RB = 0.8 x EXT (Brennan 90 deg bend rule, 1 STEP size); catalog FLANGE-p006-t01 L1 / L2 / A/F = record | OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions | MODEL: bent-tube elbow = male JIC end piece (MS33656J chain per dash from the 2403 table, round body BODYR = hex corner radius, hex HEXB over HEXL behind the JIC end) + tube (circular sweep TUBEOD along line - arc RB - line) + code 62 flange head (FLG62_MEAS by flange size: thickness, face O-ring groove; head OD = O) + one through bore TUBEID; the tube starts inside the hex body at the JIC end length and ends in the hub; braze fillets and chamfers NOT modelled; SAE code 62 flange head -32: head OD 3.125 / thickness 0.495 / groove OD 2.490 = Brennan Flange catalog table 3300-62 A / D / H (user Q-CODE62-CAT 2026-10-21); groove I.D. 2.180 / depth 0.11 = the code 61 -32 groove (FLG61_MEAS; ASSUMED: measured code 62 grooves -08 / -12 = code 61); edge chamfers not modelled; flange head with its braze hub (round, dia HUBD, from the head back face to HUBL behind the flange face; Brennan CAD geometry); the tube ends 0.05 inside the hub; the head bore is the tube bore (Brennan: 7 deg flare at the face, not modelled)</t>
         </is>
       </c>
-      <c r="AZ34" t="inlineStr">
+      <c r="AZ36" t="inlineStr">
         <is>
           <t xml:space="preserve">Brennan record 1804-32-32: L1 5.79 L2 5.31 AF 2.75 JT 0.63 GT 1.333 AFL 3.125 EFL 0.495 BFL 2.49 DFL 2.618 FFL 1.496 DRILLFL 1.693 TOD 2.087 EXT 3.814 (codes: README s2). </t>
         </is>
       </c>
-      <c r="BA34" t="inlineStr">
+      <c r="BA36" t="inlineStr">
         <is>
           <t>1804-32-32-Tube</t>
         </is>

</xml_diff>